<commit_message>
made some changes to context upserts trying to get acs locked in
</commit_message>
<xml_diff>
--- a/nvi_etl/survey/conf/nvi_answer_key_20260316.xlsx
+++ b/nvi_etl/survey/conf/nvi_answer_key_20260316.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\mike\2_responsibilities\nvi_etl\nvi_etl\survey\conf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3E8025B-5365-4FC6-B6D5-CF2E8400D767}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9010E939-80D2-41E7-B9BD-3279ACA84ACB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2880" yWindow="2880" windowWidth="19200" windowHeight="11710" xr2:uid="{E6AADBC4-36D9-4E0B-9CAE-3CD032CDA67A}"/>
+    <workbookView xWindow="3220" yWindow="3220" windowWidth="19200" windowHeight="11710" xr2:uid="{E6AADBC4-36D9-4E0B-9CAE-3CD032CDA67A}"/>
   </bookViews>
   <sheets>
     <sheet name="indicator_main" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">indicator_main!$A$1:$T$730</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">indicator_main!$A$1:$T$721</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6221" uniqueCount="743">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6149" uniqueCount="742">
   <si>
     <t>indicator_include</t>
   </si>
@@ -2266,9 +2266,6 @@
   </si>
   <si>
     <t>Have you wanted to move somewhere else in the city but not been able to find housing that you could afford?</t>
-  </si>
-  <si>
-    <t>Have financial concerns prevented you or someone in your family from getting the level of healthcare or medicine that you need?</t>
   </si>
   <si>
     <t>survey_question_type</t>
@@ -2872,15 +2869,7 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="15">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF3F3F3"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="14">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -3324,7 +3313,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1DEFEB3D-797E-4D61-9833-8A6B2512670D}">
   <sheetPr codeName="Sheet1" filterMode="1"/>
-  <dimension ref="A1:U730"/>
+  <dimension ref="A1:U721"/>
   <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="15.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="2" width="25.453125" style="3" customWidth="1"/>
@@ -3409,7 +3398,7 @@
         <v>11</v>
       </c>
       <c r="U1" s="15" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
     </row>
     <row r="2" spans="1:21" ht="18" hidden="1" x14ac:dyDescent="0.45">
@@ -6412,7 +6401,7 @@
       </c>
       <c r="M49" s="2"/>
       <c r="N49" s="2" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
       <c r="O49" s="2" t="s">
         <v>508</v>
@@ -22118,7 +22107,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="304" spans="1:21" ht="18" x14ac:dyDescent="0.45">
+    <row r="304" spans="1:21" ht="18" hidden="1" x14ac:dyDescent="0.45">
       <c r="A304" s="2">
         <v>62</v>
       </c>
@@ -22177,7 +22166,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="305" spans="1:21" ht="18" x14ac:dyDescent="0.45">
+    <row r="305" spans="1:21" ht="18" hidden="1" x14ac:dyDescent="0.45">
       <c r="A305" s="2">
         <v>62</v>
       </c>
@@ -23220,7 +23209,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="322" spans="1:21" ht="18" x14ac:dyDescent="0.45">
+    <row r="322" spans="1:21" ht="18" hidden="1" x14ac:dyDescent="0.45">
       <c r="A322" s="2">
         <v>62</v>
       </c>
@@ -23283,7 +23272,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="323" spans="1:21" ht="18" x14ac:dyDescent="0.45">
+    <row r="323" spans="1:21" ht="18" hidden="1" x14ac:dyDescent="0.45">
       <c r="A323" s="2">
         <v>62</v>
       </c>
@@ -37472,7 +37461,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="560" spans="1:21" ht="18" hidden="1" x14ac:dyDescent="0.45">
+    <row r="560" spans="1:21" ht="18" x14ac:dyDescent="0.45">
       <c r="A560" s="2">
         <v>83</v>
       </c>
@@ -37535,7 +37524,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="561" spans="1:21" ht="18" hidden="1" x14ac:dyDescent="0.45">
+    <row r="561" spans="1:21" ht="18" x14ac:dyDescent="0.45">
       <c r="A561" s="2">
         <v>83</v>
       </c>
@@ -37598,7 +37587,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="562" spans="1:21" ht="18" hidden="1" x14ac:dyDescent="0.45">
+    <row r="562" spans="1:21" ht="18" x14ac:dyDescent="0.45">
       <c r="A562" s="2">
         <v>83</v>
       </c>
@@ -44806,35 +44795,35 @@
         <v>1</v>
       </c>
       <c r="D685" s="2" t="s">
-        <v>346</v>
+        <v>548</v>
       </c>
       <c r="E685" s="2">
-        <v>3</v>
+        <v>29</v>
       </c>
       <c r="F685" s="2" t="s">
-        <v>591</v>
+        <v>621</v>
       </c>
       <c r="G685" s="2" t="s">
-        <v>740</v>
-      </c>
-      <c r="H685" s="7" t="s">
-        <v>124</v>
+        <v>701</v>
+      </c>
+      <c r="H685" s="2" t="s">
+        <v>549</v>
       </c>
       <c r="I685" s="2">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J685" s="2">
-        <v>16</v>
+        <v>177</v>
       </c>
       <c r="K685" s="7">
-        <v>36</v>
+        <v>179</v>
       </c>
       <c r="L685" s="2" t="b">
         <v>1</v>
       </c>
       <c r="M685" s="2"/>
       <c r="N685" s="2" t="s">
-        <v>348</v>
+        <v>553</v>
       </c>
       <c r="O685" s="2" t="s">
         <v>15</v>
@@ -44865,35 +44854,35 @@
         <v>1</v>
       </c>
       <c r="D686" s="2" t="s">
-        <v>346</v>
+        <v>548</v>
       </c>
       <c r="E686" s="2">
-        <v>3</v>
+        <v>29</v>
       </c>
       <c r="F686" s="2" t="s">
-        <v>591</v>
+        <v>621</v>
       </c>
       <c r="G686" s="2" t="s">
-        <v>740</v>
-      </c>
-      <c r="H686" s="7" t="s">
-        <v>122</v>
+        <v>701</v>
+      </c>
+      <c r="H686" s="2" t="s">
+        <v>287</v>
       </c>
       <c r="I686" s="2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J686" s="2">
-        <v>16</v>
+        <v>177</v>
       </c>
       <c r="K686" s="7">
-        <v>37</v>
+        <v>135</v>
       </c>
       <c r="L686" s="2" t="b">
         <v>1</v>
       </c>
       <c r="M686" s="2"/>
       <c r="N686" s="2" t="s">
-        <v>348</v>
+        <v>553</v>
       </c>
       <c r="O686" s="2" t="s">
         <v>15</v>
@@ -44924,35 +44913,35 @@
         <v>1</v>
       </c>
       <c r="D687" s="2" t="s">
-        <v>346</v>
+        <v>548</v>
       </c>
       <c r="E687" s="2">
-        <v>3</v>
+        <v>29</v>
       </c>
       <c r="F687" s="2" t="s">
-        <v>591</v>
+        <v>621</v>
       </c>
       <c r="G687" s="2" t="s">
-        <v>740</v>
-      </c>
-      <c r="H687" s="7" t="s">
-        <v>125</v>
+        <v>701</v>
+      </c>
+      <c r="H687" s="2" t="s">
+        <v>289</v>
       </c>
       <c r="I687" s="2">
         <v>3</v>
       </c>
       <c r="J687" s="2">
-        <v>16</v>
+        <v>177</v>
       </c>
       <c r="K687" s="7">
-        <v>39</v>
+        <v>134</v>
       </c>
       <c r="L687" s="2" t="b">
         <v>1</v>
       </c>
       <c r="M687" s="2"/>
       <c r="N687" s="2" t="s">
-        <v>348</v>
+        <v>553</v>
       </c>
       <c r="O687" s="2" t="s">
         <v>15</v>
@@ -44983,35 +44972,35 @@
         <v>1</v>
       </c>
       <c r="D688" s="2" t="s">
-        <v>346</v>
+        <v>548</v>
       </c>
       <c r="E688" s="2">
-        <v>3</v>
+        <v>29</v>
       </c>
       <c r="F688" s="2" t="s">
-        <v>591</v>
+        <v>621</v>
       </c>
       <c r="G688" s="2" t="s">
-        <v>739</v>
-      </c>
-      <c r="H688" s="7" t="s">
-        <v>124</v>
+        <v>701</v>
+      </c>
+      <c r="H688" s="2" t="s">
+        <v>550</v>
       </c>
       <c r="I688" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J688" s="2">
-        <v>17</v>
+        <v>177</v>
       </c>
       <c r="K688" s="7">
-        <v>36</v>
+        <v>180</v>
       </c>
       <c r="L688" s="2" t="b">
         <v>1</v>
       </c>
       <c r="M688" s="2"/>
       <c r="N688" s="2" t="s">
-        <v>349</v>
+        <v>553</v>
       </c>
       <c r="O688" s="2" t="s">
         <v>15</v>
@@ -45042,35 +45031,35 @@
         <v>1</v>
       </c>
       <c r="D689" s="2" t="s">
-        <v>346</v>
+        <v>548</v>
       </c>
       <c r="E689" s="2">
-        <v>3</v>
+        <v>29</v>
       </c>
       <c r="F689" s="2" t="s">
-        <v>591</v>
+        <v>621</v>
       </c>
       <c r="G689" s="2" t="s">
-        <v>739</v>
-      </c>
-      <c r="H689" s="7" t="s">
-        <v>122</v>
+        <v>701</v>
+      </c>
+      <c r="H689" s="2" t="s">
+        <v>551</v>
       </c>
       <c r="I689" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J689" s="2">
-        <v>17</v>
+        <v>177</v>
       </c>
       <c r="K689" s="7">
-        <v>37</v>
+        <v>181</v>
       </c>
       <c r="L689" s="2" t="b">
         <v>1</v>
       </c>
       <c r="M689" s="2"/>
       <c r="N689" s="2" t="s">
-        <v>349</v>
+        <v>553</v>
       </c>
       <c r="O689" s="2" t="s">
         <v>15</v>
@@ -45101,35 +45090,35 @@
         <v>1</v>
       </c>
       <c r="D690" s="2" t="s">
-        <v>346</v>
+        <v>548</v>
       </c>
       <c r="E690" s="2">
-        <v>3</v>
+        <v>29</v>
       </c>
       <c r="F690" s="2" t="s">
-        <v>591</v>
+        <v>621</v>
       </c>
       <c r="G690" s="2" t="s">
-        <v>739</v>
-      </c>
-      <c r="H690" s="7" t="s">
-        <v>125</v>
+        <v>702</v>
+      </c>
+      <c r="H690" s="2" t="s">
+        <v>549</v>
       </c>
       <c r="I690" s="2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J690" s="2">
-        <v>17</v>
+        <v>178</v>
       </c>
       <c r="K690" s="7">
-        <v>39</v>
+        <v>179</v>
       </c>
       <c r="L690" s="2" t="b">
         <v>1</v>
       </c>
       <c r="M690" s="2"/>
       <c r="N690" s="2" t="s">
-        <v>349</v>
+        <v>554</v>
       </c>
       <c r="O690" s="2" t="s">
         <v>15</v>
@@ -45160,35 +45149,35 @@
         <v>1</v>
       </c>
       <c r="D691" s="2" t="s">
-        <v>346</v>
+        <v>548</v>
       </c>
       <c r="E691" s="2">
-        <v>3</v>
+        <v>29</v>
       </c>
       <c r="F691" s="2" t="s">
-        <v>591</v>
+        <v>621</v>
       </c>
       <c r="G691" s="2" t="s">
-        <v>738</v>
-      </c>
-      <c r="H691" s="7" t="s">
-        <v>124</v>
+        <v>702</v>
+      </c>
+      <c r="H691" s="2" t="s">
+        <v>287</v>
       </c>
       <c r="I691" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J691" s="2">
-        <v>18</v>
+        <v>178</v>
       </c>
       <c r="K691" s="7">
-        <v>36</v>
+        <v>135</v>
       </c>
       <c r="L691" s="2" t="b">
         <v>1</v>
       </c>
       <c r="M691" s="2"/>
       <c r="N691" s="2" t="s">
-        <v>347</v>
+        <v>554</v>
       </c>
       <c r="O691" s="2" t="s">
         <v>15</v>
@@ -45219,35 +45208,35 @@
         <v>1</v>
       </c>
       <c r="D692" s="2" t="s">
-        <v>346</v>
+        <v>548</v>
       </c>
       <c r="E692" s="2">
+        <v>29</v>
+      </c>
+      <c r="F692" s="2" t="s">
+        <v>621</v>
+      </c>
+      <c r="G692" s="2" t="s">
+        <v>702</v>
+      </c>
+      <c r="H692" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="I692" s="2">
         <v>3</v>
       </c>
-      <c r="F692" s="2" t="s">
-        <v>591</v>
-      </c>
-      <c r="G692" s="2" t="s">
-        <v>738</v>
-      </c>
-      <c r="H692" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="I692" s="2">
-        <v>2</v>
-      </c>
       <c r="J692" s="2">
-        <v>18</v>
+        <v>178</v>
       </c>
       <c r="K692" s="7">
-        <v>37</v>
+        <v>134</v>
       </c>
       <c r="L692" s="2" t="b">
         <v>1</v>
       </c>
       <c r="M692" s="2"/>
       <c r="N692" s="2" t="s">
-        <v>347</v>
+        <v>554</v>
       </c>
       <c r="O692" s="2" t="s">
         <v>15</v>
@@ -45278,35 +45267,35 @@
         <v>1</v>
       </c>
       <c r="D693" s="2" t="s">
-        <v>346</v>
+        <v>548</v>
       </c>
       <c r="E693" s="2">
-        <v>3</v>
+        <v>29</v>
       </c>
       <c r="F693" s="2" t="s">
-        <v>591</v>
+        <v>621</v>
       </c>
       <c r="G693" s="2" t="s">
-        <v>738</v>
-      </c>
-      <c r="H693" s="7" t="s">
-        <v>125</v>
+        <v>702</v>
+      </c>
+      <c r="H693" s="2" t="s">
+        <v>550</v>
       </c>
       <c r="I693" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J693" s="2">
-        <v>18</v>
+        <v>178</v>
       </c>
       <c r="K693" s="7">
-        <v>39</v>
+        <v>180</v>
       </c>
       <c r="L693" s="2" t="b">
         <v>1</v>
       </c>
       <c r="M693" s="2"/>
       <c r="N693" s="2" t="s">
-        <v>347</v>
+        <v>554</v>
       </c>
       <c r="O693" s="2" t="s">
         <v>15</v>
@@ -45346,26 +45335,26 @@
         <v>621</v>
       </c>
       <c r="G694" s="2" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="H694" s="2" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="I694" s="2">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J694" s="2">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="K694" s="7">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="L694" s="2" t="b">
         <v>1</v>
       </c>
       <c r="M694" s="2"/>
       <c r="N694" s="2" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="O694" s="2" t="s">
         <v>15</v>
@@ -45405,26 +45394,26 @@
         <v>621</v>
       </c>
       <c r="G695" s="2" t="s">
-        <v>701</v>
+        <v>703</v>
       </c>
       <c r="H695" s="2" t="s">
-        <v>287</v>
+        <v>549</v>
       </c>
       <c r="I695" s="2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J695" s="2">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="K695" s="7">
-        <v>135</v>
+        <v>179</v>
       </c>
       <c r="L695" s="2" t="b">
         <v>1</v>
       </c>
       <c r="M695" s="2"/>
       <c r="N695" s="2" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="O695" s="2" t="s">
         <v>15</v>
@@ -45464,26 +45453,26 @@
         <v>621</v>
       </c>
       <c r="G696" s="2" t="s">
-        <v>701</v>
+        <v>703</v>
       </c>
       <c r="H696" s="2" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="I696" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J696" s="2">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="K696" s="7">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="L696" s="2" t="b">
         <v>1</v>
       </c>
       <c r="M696" s="2"/>
       <c r="N696" s="2" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="O696" s="2" t="s">
         <v>15</v>
@@ -45523,26 +45512,26 @@
         <v>621</v>
       </c>
       <c r="G697" s="2" t="s">
-        <v>701</v>
+        <v>703</v>
       </c>
       <c r="H697" s="2" t="s">
-        <v>550</v>
+        <v>289</v>
       </c>
       <c r="I697" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J697" s="2">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="K697" s="7">
-        <v>180</v>
+        <v>134</v>
       </c>
       <c r="L697" s="2" t="b">
         <v>1</v>
       </c>
       <c r="M697" s="2"/>
       <c r="N697" s="2" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="O697" s="2" t="s">
         <v>15</v>
@@ -45582,26 +45571,26 @@
         <v>621</v>
       </c>
       <c r="G698" s="2" t="s">
-        <v>701</v>
+        <v>703</v>
       </c>
       <c r="H698" s="2" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="I698" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J698" s="2">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="K698" s="7">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="L698" s="2" t="b">
         <v>1</v>
       </c>
       <c r="M698" s="2"/>
       <c r="N698" s="2" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="O698" s="2" t="s">
         <v>15</v>
@@ -45641,26 +45630,26 @@
         <v>621</v>
       </c>
       <c r="G699" s="2" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="H699" s="2" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="I699" s="2">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J699" s="2">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="K699" s="7">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="L699" s="2" t="b">
         <v>1</v>
       </c>
       <c r="M699" s="2"/>
       <c r="N699" s="2" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="O699" s="2" t="s">
         <v>15</v>
@@ -45700,26 +45689,26 @@
         <v>621</v>
       </c>
       <c r="G700" s="2" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="H700" s="2" t="s">
-        <v>287</v>
+        <v>549</v>
       </c>
       <c r="I700" s="2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J700" s="2">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="K700" s="7">
-        <v>135</v>
+        <v>179</v>
       </c>
       <c r="L700" s="2" t="b">
         <v>1</v>
       </c>
       <c r="M700" s="2"/>
       <c r="N700" s="2" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="O700" s="2" t="s">
         <v>15</v>
@@ -45759,26 +45748,26 @@
         <v>621</v>
       </c>
       <c r="G701" s="2" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="H701" s="2" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="I701" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J701" s="2">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="K701" s="7">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="L701" s="2" t="b">
         <v>1</v>
       </c>
       <c r="M701" s="2"/>
       <c r="N701" s="2" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="O701" s="2" t="s">
         <v>15</v>
@@ -45818,26 +45807,26 @@
         <v>621</v>
       </c>
       <c r="G702" s="2" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="H702" s="2" t="s">
-        <v>550</v>
+        <v>289</v>
       </c>
       <c r="I702" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J702" s="2">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="K702" s="7">
-        <v>180</v>
+        <v>134</v>
       </c>
       <c r="L702" s="2" t="b">
         <v>1</v>
       </c>
       <c r="M702" s="2"/>
       <c r="N702" s="2" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="O702" s="2" t="s">
         <v>15</v>
@@ -45877,26 +45866,26 @@
         <v>621</v>
       </c>
       <c r="G703" s="2" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="H703" s="2" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="I703" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J703" s="2">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="K703" s="7">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="L703" s="2" t="b">
         <v>1</v>
       </c>
       <c r="M703" s="2"/>
       <c r="N703" s="2" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="O703" s="2" t="s">
         <v>15</v>
@@ -45936,26 +45925,26 @@
         <v>621</v>
       </c>
       <c r="G704" s="2" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="H704" s="2" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="I704" s="2">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J704" s="2">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="K704" s="7">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="L704" s="2" t="b">
         <v>1</v>
       </c>
       <c r="M704" s="2"/>
       <c r="N704" s="2" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="O704" s="2" t="s">
         <v>15</v>
@@ -45995,26 +45984,26 @@
         <v>621</v>
       </c>
       <c r="G705" s="2" t="s">
-        <v>703</v>
+        <v>705</v>
       </c>
       <c r="H705" s="2" t="s">
-        <v>287</v>
+        <v>549</v>
       </c>
       <c r="I705" s="2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J705" s="2">
+        <v>181</v>
+      </c>
+      <c r="K705" s="7">
         <v>179</v>
-      </c>
-      <c r="K705" s="7">
-        <v>135</v>
       </c>
       <c r="L705" s="2" t="b">
         <v>1</v>
       </c>
       <c r="M705" s="2"/>
       <c r="N705" s="2" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="O705" s="2" t="s">
         <v>15</v>
@@ -46054,26 +46043,26 @@
         <v>621</v>
       </c>
       <c r="G706" s="2" t="s">
-        <v>703</v>
+        <v>705</v>
       </c>
       <c r="H706" s="2" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="I706" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J706" s="2">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="K706" s="7">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="L706" s="2" t="b">
         <v>1</v>
       </c>
       <c r="M706" s="2"/>
       <c r="N706" s="2" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="O706" s="2" t="s">
         <v>15</v>
@@ -46113,26 +46102,26 @@
         <v>621</v>
       </c>
       <c r="G707" s="2" t="s">
-        <v>703</v>
+        <v>705</v>
       </c>
       <c r="H707" s="2" t="s">
-        <v>550</v>
+        <v>289</v>
       </c>
       <c r="I707" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J707" s="2">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="K707" s="7">
-        <v>180</v>
+        <v>134</v>
       </c>
       <c r="L707" s="2" t="b">
         <v>1</v>
       </c>
       <c r="M707" s="2"/>
       <c r="N707" s="2" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="O707" s="2" t="s">
         <v>15</v>
@@ -46172,26 +46161,26 @@
         <v>621</v>
       </c>
       <c r="G708" s="2" t="s">
-        <v>703</v>
+        <v>705</v>
       </c>
       <c r="H708" s="2" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="I708" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J708" s="2">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="K708" s="7">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="L708" s="2" t="b">
         <v>1</v>
       </c>
       <c r="M708" s="2"/>
       <c r="N708" s="2" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="O708" s="2" t="s">
         <v>15</v>
@@ -46231,26 +46220,26 @@
         <v>621</v>
       </c>
       <c r="G709" s="2" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="H709" s="2" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="I709" s="2">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J709" s="2">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="K709" s="7">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="L709" s="2" t="b">
         <v>1</v>
       </c>
       <c r="M709" s="2"/>
       <c r="N709" s="2" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="O709" s="2" t="s">
         <v>15</v>
@@ -46278,38 +46267,38 @@
         <v>0</v>
       </c>
       <c r="C710" s="2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D710" s="2" t="s">
-        <v>548</v>
+        <v>558</v>
       </c>
       <c r="E710" s="2">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F710" s="2" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="G710" s="2" t="s">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="H710" s="2" t="s">
-        <v>287</v>
+        <v>528</v>
       </c>
       <c r="I710" s="2">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J710" s="2">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="K710" s="7">
-        <v>135</v>
+        <v>16</v>
       </c>
       <c r="L710" s="2" t="b">
         <v>1</v>
       </c>
       <c r="M710" s="2"/>
       <c r="N710" s="2" t="s">
-        <v>556</v>
+        <v>559</v>
       </c>
       <c r="O710" s="2" t="s">
         <v>15</v>
@@ -46340,35 +46329,35 @@
         <v>1</v>
       </c>
       <c r="D711" s="2" t="s">
-        <v>548</v>
+        <v>558</v>
       </c>
       <c r="E711" s="2">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F711" s="2" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="G711" s="2" t="s">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="H711" s="2" t="s">
-        <v>289</v>
+        <v>25</v>
       </c>
       <c r="I711" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J711" s="2">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="K711" s="7">
-        <v>134</v>
+        <v>1</v>
       </c>
       <c r="L711" s="2" t="b">
         <v>1</v>
       </c>
       <c r="M711" s="2"/>
       <c r="N711" s="2" t="s">
-        <v>556</v>
+        <v>559</v>
       </c>
       <c r="O711" s="2" t="s">
         <v>15</v>
@@ -46399,35 +46388,35 @@
         <v>1</v>
       </c>
       <c r="D712" s="2" t="s">
-        <v>548</v>
+        <v>558</v>
       </c>
       <c r="E712" s="2">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F712" s="2" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="G712" s="2" t="s">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="H712" s="2" t="s">
-        <v>550</v>
+        <v>24</v>
       </c>
       <c r="I712" s="2">
         <v>2</v>
       </c>
       <c r="J712" s="2">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="K712" s="7">
-        <v>180</v>
+        <v>2</v>
       </c>
       <c r="L712" s="2" t="b">
         <v>1</v>
       </c>
       <c r="M712" s="2"/>
       <c r="N712" s="2" t="s">
-        <v>556</v>
+        <v>559</v>
       </c>
       <c r="O712" s="2" t="s">
         <v>15</v>
@@ -46458,35 +46447,35 @@
         <v>1</v>
       </c>
       <c r="D713" s="2" t="s">
-        <v>548</v>
+        <v>558</v>
       </c>
       <c r="E713" s="2">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F713" s="2" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="G713" s="2" t="s">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="H713" s="2" t="s">
-        <v>551</v>
+        <v>23</v>
       </c>
       <c r="I713" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J713" s="2">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="K713" s="7">
-        <v>181</v>
+        <v>3</v>
       </c>
       <c r="L713" s="2" t="b">
         <v>1</v>
       </c>
       <c r="M713" s="2"/>
       <c r="N713" s="2" t="s">
-        <v>556</v>
+        <v>559</v>
       </c>
       <c r="O713" s="2" t="s">
         <v>15</v>
@@ -46517,35 +46506,35 @@
         <v>1</v>
       </c>
       <c r="D714" s="2" t="s">
-        <v>548</v>
+        <v>558</v>
       </c>
       <c r="E714" s="2">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F714" s="2" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="G714" s="2" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="H714" s="2" t="s">
-        <v>549</v>
+        <v>21</v>
       </c>
       <c r="I714" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J714" s="2">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="K714" s="7">
-        <v>179</v>
+        <v>4</v>
       </c>
       <c r="L714" s="2" t="b">
         <v>1</v>
       </c>
       <c r="M714" s="2"/>
       <c r="N714" s="2" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
       <c r="O714" s="2" t="s">
         <v>15</v>
@@ -46573,38 +46562,38 @@
         <v>0</v>
       </c>
       <c r="C715" s="2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D715" s="2" t="s">
-        <v>548</v>
+        <v>558</v>
       </c>
       <c r="E715" s="2">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F715" s="2" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="G715" s="2" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
       <c r="H715" s="2" t="s">
-        <v>287</v>
+        <v>561</v>
       </c>
       <c r="I715" s="2">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J715" s="2">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="K715" s="7">
-        <v>135</v>
+        <v>16</v>
       </c>
       <c r="L715" s="2" t="b">
         <v>1</v>
       </c>
       <c r="M715" s="2"/>
       <c r="N715" s="2" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="O715" s="2" t="s">
         <v>15</v>
@@ -46635,35 +46624,35 @@
         <v>1</v>
       </c>
       <c r="D716" s="2" t="s">
-        <v>548</v>
+        <v>558</v>
       </c>
       <c r="E716" s="2">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F716" s="2" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="G716" s="2" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
       <c r="H716" s="2" t="s">
-        <v>289</v>
+        <v>25</v>
       </c>
       <c r="I716" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J716" s="2">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="K716" s="7">
-        <v>134</v>
+        <v>1</v>
       </c>
       <c r="L716" s="2" t="b">
         <v>1</v>
       </c>
       <c r="M716" s="2"/>
       <c r="N716" s="2" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="O716" s="2" t="s">
         <v>15</v>
@@ -46694,35 +46683,35 @@
         <v>1</v>
       </c>
       <c r="D717" s="2" t="s">
-        <v>548</v>
+        <v>558</v>
       </c>
       <c r="E717" s="2">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F717" s="2" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="G717" s="2" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
       <c r="H717" s="2" t="s">
-        <v>550</v>
+        <v>24</v>
       </c>
       <c r="I717" s="2">
         <v>2</v>
       </c>
       <c r="J717" s="2">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="K717" s="7">
-        <v>180</v>
+        <v>2</v>
       </c>
       <c r="L717" s="2" t="b">
         <v>1</v>
       </c>
       <c r="M717" s="2"/>
       <c r="N717" s="2" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="O717" s="2" t="s">
         <v>15</v>
@@ -46753,35 +46742,35 @@
         <v>1</v>
       </c>
       <c r="D718" s="2" t="s">
-        <v>548</v>
+        <v>558</v>
       </c>
       <c r="E718" s="2">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F718" s="2" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="G718" s="2" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
       <c r="H718" s="2" t="s">
-        <v>551</v>
+        <v>23</v>
       </c>
       <c r="I718" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J718" s="2">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="K718" s="7">
-        <v>181</v>
+        <v>3</v>
       </c>
       <c r="L718" s="2" t="b">
         <v>1</v>
       </c>
       <c r="M718" s="2"/>
       <c r="N718" s="2" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="O718" s="2" t="s">
         <v>15</v>
@@ -46809,7 +46798,7 @@
         <v>0</v>
       </c>
       <c r="C719" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D719" s="2" t="s">
         <v>558</v>
@@ -46821,26 +46810,26 @@
         <v>622</v>
       </c>
       <c r="G719" s="2" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="H719" s="2" t="s">
-        <v>528</v>
+        <v>21</v>
       </c>
       <c r="I719" s="2">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J719" s="2">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K719" s="7">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="L719" s="2" t="b">
         <v>1</v>
       </c>
       <c r="M719" s="2"/>
       <c r="N719" s="2" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="O719" s="2" t="s">
         <v>15</v>
@@ -46871,38 +46860,34 @@
         <v>1</v>
       </c>
       <c r="D720" s="2" t="s">
-        <v>558</v>
-      </c>
-      <c r="E720" s="2">
-        <v>30</v>
-      </c>
-      <c r="F720" s="2" t="s">
-        <v>622</v>
-      </c>
+        <v>552</v>
+      </c>
+      <c r="E720" s="2"/>
+      <c r="F720" s="2"/>
       <c r="G720" s="2" t="s">
-        <v>706</v>
+        <v>708</v>
       </c>
       <c r="H720" s="2" t="s">
-        <v>25</v>
+        <v>124</v>
       </c>
       <c r="I720" s="2">
         <v>1</v>
       </c>
       <c r="J720" s="2">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="K720" s="7">
-        <v>1</v>
+        <v>36</v>
       </c>
       <c r="L720" s="2" t="b">
         <v>1</v>
       </c>
       <c r="M720" s="2"/>
       <c r="N720" s="2" t="s">
-        <v>559</v>
+        <v>552</v>
       </c>
       <c r="O720" s="2" t="s">
-        <v>15</v>
+        <v>509</v>
       </c>
       <c r="P720" s="6" t="s">
         <v>521</v>
@@ -46930,38 +46915,34 @@
         <v>1</v>
       </c>
       <c r="D721" s="2" t="s">
-        <v>558</v>
-      </c>
-      <c r="E721" s="2">
-        <v>30</v>
-      </c>
-      <c r="F721" s="2" t="s">
-        <v>622</v>
-      </c>
+        <v>552</v>
+      </c>
+      <c r="E721" s="2"/>
+      <c r="F721" s="2"/>
       <c r="G721" s="2" t="s">
-        <v>706</v>
+        <v>708</v>
       </c>
       <c r="H721" s="2" t="s">
-        <v>24</v>
+        <v>122</v>
       </c>
       <c r="I721" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J721" s="2">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="K721" s="7">
-        <v>2</v>
+        <v>37</v>
       </c>
       <c r="L721" s="2" t="b">
         <v>1</v>
       </c>
       <c r="M721" s="2"/>
       <c r="N721" s="2" t="s">
-        <v>559</v>
+        <v>552</v>
       </c>
       <c r="O721" s="2" t="s">
-        <v>15</v>
+        <v>509</v>
       </c>
       <c r="P721" s="6" t="s">
         <v>521</v>
@@ -46980,611 +46961,83 @@
         <v>4</v>
       </c>
     </row>
-    <row r="722" spans="1:21" ht="18" hidden="1" x14ac:dyDescent="0.45">
-      <c r="A722" s="2"/>
-      <c r="B722" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="C722" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="D722" s="2" t="s">
-        <v>558</v>
-      </c>
-      <c r="E722" s="2">
-        <v>30</v>
-      </c>
-      <c r="F722" s="2" t="s">
-        <v>622</v>
-      </c>
-      <c r="G722" s="2" t="s">
-        <v>706</v>
-      </c>
-      <c r="H722" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="I722" s="2">
-        <v>3</v>
-      </c>
-      <c r="J722" s="2">
-        <v>182</v>
-      </c>
-      <c r="K722" s="7">
-        <v>3</v>
-      </c>
-      <c r="L722" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="M722" s="2"/>
-      <c r="N722" s="2" t="s">
-        <v>559</v>
-      </c>
-      <c r="O722" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="P722" s="6" t="s">
-        <v>521</v>
-      </c>
-      <c r="Q722" s="2"/>
-      <c r="R722" s="2" t="s">
-        <v>525</v>
-      </c>
-      <c r="S722" s="9">
-        <v>45658</v>
-      </c>
-      <c r="T722" s="14">
-        <v>72686</v>
-      </c>
-      <c r="U722" s="16">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="723" spans="1:21" ht="18" hidden="1" x14ac:dyDescent="0.45">
-      <c r="A723" s="2"/>
-      <c r="B723" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="C723" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="D723" s="2" t="s">
-        <v>558</v>
-      </c>
-      <c r="E723" s="2">
-        <v>30</v>
-      </c>
-      <c r="F723" s="2" t="s">
-        <v>622</v>
-      </c>
-      <c r="G723" s="2" t="s">
-        <v>706</v>
-      </c>
-      <c r="H723" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="I723" s="2">
-        <v>4</v>
-      </c>
-      <c r="J723" s="2">
-        <v>182</v>
-      </c>
-      <c r="K723" s="7">
-        <v>4</v>
-      </c>
-      <c r="L723" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="M723" s="2"/>
-      <c r="N723" s="2" t="s">
-        <v>559</v>
-      </c>
-      <c r="O723" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="P723" s="6" t="s">
-        <v>521</v>
-      </c>
-      <c r="Q723" s="2"/>
-      <c r="R723" s="2" t="s">
-        <v>525</v>
-      </c>
-      <c r="S723" s="9">
-        <v>45658</v>
-      </c>
-      <c r="T723" s="14">
-        <v>72686</v>
-      </c>
-      <c r="U723" s="16">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="724" spans="1:21" ht="18" hidden="1" x14ac:dyDescent="0.45">
-      <c r="A724" s="2"/>
-      <c r="B724" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="C724" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="D724" s="2" t="s">
-        <v>558</v>
-      </c>
-      <c r="E724" s="2">
-        <v>30</v>
-      </c>
-      <c r="F724" s="2" t="s">
-        <v>622</v>
-      </c>
-      <c r="G724" s="2" t="s">
-        <v>707</v>
-      </c>
-      <c r="H724" s="2" t="s">
-        <v>561</v>
-      </c>
-      <c r="I724" s="2">
-        <v>0</v>
-      </c>
-      <c r="J724" s="2">
-        <v>183</v>
-      </c>
-      <c r="K724" s="7">
-        <v>16</v>
-      </c>
-      <c r="L724" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="M724" s="2"/>
-      <c r="N724" s="2" t="s">
-        <v>560</v>
-      </c>
-      <c r="O724" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="P724" s="6" t="s">
-        <v>521</v>
-      </c>
-      <c r="Q724" s="2"/>
-      <c r="R724" s="2" t="s">
-        <v>525</v>
-      </c>
-      <c r="S724" s="9">
-        <v>45658</v>
-      </c>
-      <c r="T724" s="14">
-        <v>72686</v>
-      </c>
-      <c r="U724" s="16">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="725" spans="1:21" ht="18" hidden="1" x14ac:dyDescent="0.45">
-      <c r="A725" s="2"/>
-      <c r="B725" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="C725" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="D725" s="2" t="s">
-        <v>558</v>
-      </c>
-      <c r="E725" s="2">
-        <v>30</v>
-      </c>
-      <c r="F725" s="2" t="s">
-        <v>622</v>
-      </c>
-      <c r="G725" s="2" t="s">
-        <v>707</v>
-      </c>
-      <c r="H725" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="I725" s="2">
-        <v>1</v>
-      </c>
-      <c r="J725" s="2">
-        <v>183</v>
-      </c>
-      <c r="K725" s="7">
-        <v>1</v>
-      </c>
-      <c r="L725" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="M725" s="2"/>
-      <c r="N725" s="2" t="s">
-        <v>560</v>
-      </c>
-      <c r="O725" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="P725" s="6" t="s">
-        <v>521</v>
-      </c>
-      <c r="Q725" s="2"/>
-      <c r="R725" s="2" t="s">
-        <v>525</v>
-      </c>
-      <c r="S725" s="9">
-        <v>45658</v>
-      </c>
-      <c r="T725" s="14">
-        <v>72686</v>
-      </c>
-      <c r="U725" s="16">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="726" spans="1:21" ht="18" hidden="1" x14ac:dyDescent="0.45">
-      <c r="A726" s="2"/>
-      <c r="B726" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="C726" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="D726" s="2" t="s">
-        <v>558</v>
-      </c>
-      <c r="E726" s="2">
-        <v>30</v>
-      </c>
-      <c r="F726" s="2" t="s">
-        <v>622</v>
-      </c>
-      <c r="G726" s="2" t="s">
-        <v>707</v>
-      </c>
-      <c r="H726" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="I726" s="2">
-        <v>2</v>
-      </c>
-      <c r="J726" s="2">
-        <v>183</v>
-      </c>
-      <c r="K726" s="7">
-        <v>2</v>
-      </c>
-      <c r="L726" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="M726" s="2"/>
-      <c r="N726" s="2" t="s">
-        <v>560</v>
-      </c>
-      <c r="O726" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="P726" s="6" t="s">
-        <v>521</v>
-      </c>
-      <c r="Q726" s="2"/>
-      <c r="R726" s="2" t="s">
-        <v>525</v>
-      </c>
-      <c r="S726" s="9">
-        <v>45658</v>
-      </c>
-      <c r="T726" s="14">
-        <v>72686</v>
-      </c>
-      <c r="U726" s="16">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="727" spans="1:21" ht="18" hidden="1" x14ac:dyDescent="0.45">
-      <c r="A727" s="2"/>
-      <c r="B727" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="C727" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="D727" s="2" t="s">
-        <v>558</v>
-      </c>
-      <c r="E727" s="2">
-        <v>30</v>
-      </c>
-      <c r="F727" s="2" t="s">
-        <v>622</v>
-      </c>
-      <c r="G727" s="2" t="s">
-        <v>707</v>
-      </c>
-      <c r="H727" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="I727" s="2">
-        <v>3</v>
-      </c>
-      <c r="J727" s="2">
-        <v>183</v>
-      </c>
-      <c r="K727" s="7">
-        <v>3</v>
-      </c>
-      <c r="L727" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="M727" s="2"/>
-      <c r="N727" s="2" t="s">
-        <v>560</v>
-      </c>
-      <c r="O727" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="P727" s="6" t="s">
-        <v>521</v>
-      </c>
-      <c r="Q727" s="2"/>
-      <c r="R727" s="2" t="s">
-        <v>525</v>
-      </c>
-      <c r="S727" s="9">
-        <v>45658</v>
-      </c>
-      <c r="T727" s="14">
-        <v>72686</v>
-      </c>
-      <c r="U727" s="16">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="728" spans="1:21" ht="18" hidden="1" x14ac:dyDescent="0.45">
-      <c r="A728" s="2"/>
-      <c r="B728" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="C728" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="D728" s="2" t="s">
-        <v>558</v>
-      </c>
-      <c r="E728" s="2">
-        <v>30</v>
-      </c>
-      <c r="F728" s="2" t="s">
-        <v>622</v>
-      </c>
-      <c r="G728" s="2" t="s">
-        <v>707</v>
-      </c>
-      <c r="H728" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="I728" s="2">
-        <v>4</v>
-      </c>
-      <c r="J728" s="2">
-        <v>183</v>
-      </c>
-      <c r="K728" s="7">
-        <v>4</v>
-      </c>
-      <c r="L728" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="M728" s="2"/>
-      <c r="N728" s="2" t="s">
-        <v>560</v>
-      </c>
-      <c r="O728" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="P728" s="6" t="s">
-        <v>521</v>
-      </c>
-      <c r="Q728" s="2"/>
-      <c r="R728" s="2" t="s">
-        <v>525</v>
-      </c>
-      <c r="S728" s="9">
-        <v>45658</v>
-      </c>
-      <c r="T728" s="14">
-        <v>72686</v>
-      </c>
-      <c r="U728" s="16">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="729" spans="1:21" ht="18" hidden="1" x14ac:dyDescent="0.45">
-      <c r="A729" s="2"/>
-      <c r="B729" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="C729" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="D729" s="2" t="s">
-        <v>552</v>
-      </c>
-      <c r="E729" s="2"/>
-      <c r="F729" s="2"/>
-      <c r="G729" s="2" t="s">
-        <v>708</v>
-      </c>
-      <c r="H729" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="I729" s="2">
-        <v>1</v>
-      </c>
-      <c r="J729" s="2">
-        <v>184</v>
-      </c>
-      <c r="K729" s="7">
-        <v>36</v>
-      </c>
-      <c r="L729" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="M729" s="2"/>
-      <c r="N729" s="2" t="s">
-        <v>552</v>
-      </c>
-      <c r="O729" s="2" t="s">
-        <v>509</v>
-      </c>
-      <c r="P729" s="6" t="s">
-        <v>521</v>
-      </c>
-      <c r="Q729" s="2"/>
-      <c r="R729" s="2" t="s">
-        <v>525</v>
-      </c>
-      <c r="S729" s="9">
-        <v>45658</v>
-      </c>
-      <c r="T729" s="14">
-        <v>72686</v>
-      </c>
-      <c r="U729" s="16">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="730" spans="1:21" ht="18" hidden="1" x14ac:dyDescent="0.45">
-      <c r="A730" s="2"/>
-      <c r="B730" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="C730" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="D730" s="2" t="s">
-        <v>552</v>
-      </c>
-      <c r="E730" s="2"/>
-      <c r="F730" s="2"/>
-      <c r="G730" s="2" t="s">
-        <v>708</v>
-      </c>
-      <c r="H730" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="I730" s="2">
-        <v>0</v>
-      </c>
-      <c r="J730" s="2">
-        <v>184</v>
-      </c>
-      <c r="K730" s="7">
-        <v>37</v>
-      </c>
-      <c r="L730" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="M730" s="2"/>
-      <c r="N730" s="2" t="s">
-        <v>552</v>
-      </c>
-      <c r="O730" s="2" t="s">
-        <v>509</v>
-      </c>
-      <c r="P730" s="6" t="s">
-        <v>521</v>
-      </c>
-      <c r="Q730" s="2"/>
-      <c r="R730" s="2" t="s">
-        <v>525</v>
-      </c>
-      <c r="S730" s="9">
-        <v>45658</v>
-      </c>
-      <c r="T730" s="14">
-        <v>72686</v>
-      </c>
-      <c r="U730" s="16">
-        <v>4</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:T730" xr:uid="{1DEFEB3D-797E-4D61-9833-8A6B2512670D}">
-    <filterColumn colId="0">
+  <autoFilter ref="A1:T721" xr:uid="{1DEFEB3D-797E-4D61-9833-8A6B2512670D}">
+    <filterColumn colId="13">
       <filters>
-        <filter val="62"/>
+        <filter val="At_Risk_Losing_Home:Needs_In_Past_12_Months"/>
       </filters>
     </filterColumn>
   </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:T642">
     <sortCondition ref="A2:A642"/>
   </sortState>
-  <conditionalFormatting sqref="A1:T1 T1:U730 A2:F305 I653:J653 G660:J730">
-    <cfRule type="expression" dxfId="14" priority="4">
+  <conditionalFormatting sqref="A1:T1 A2:F305 I653:J653 R653:T684 O653:O684 L651:L684 M654:N684 T1:U721 G660:J721 K2:K721 C306:C721 A493:B721 D661:F721 O685:P721">
+    <cfRule type="expression" dxfId="13" priority="4">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D665:E684">
-    <cfRule type="expression" dxfId="13" priority="42">
+    <cfRule type="expression" dxfId="12" priority="42">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D306:F652">
-    <cfRule type="expression" dxfId="12" priority="3">
+    <cfRule type="expression" dxfId="11" priority="3">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G671:G674">
-    <cfRule type="expression" dxfId="11" priority="41">
+    <cfRule type="expression" dxfId="10" priority="41">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:J652">
-    <cfRule type="expression" dxfId="10" priority="1">
+    <cfRule type="expression" dxfId="9" priority="1">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H675">
-    <cfRule type="expression" dxfId="9" priority="39">
+    <cfRule type="expression" dxfId="8" priority="39">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H680">
-    <cfRule type="expression" dxfId="8" priority="36">
+    <cfRule type="expression" dxfId="7" priority="36">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I670:I673">
-    <cfRule type="expression" dxfId="7" priority="35">
+    <cfRule type="expression" dxfId="6" priority="35">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I675:I678">
-    <cfRule type="expression" dxfId="6" priority="34">
+    <cfRule type="expression" dxfId="5" priority="34">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I680:I683">
-    <cfRule type="expression" dxfId="5" priority="33">
+    <cfRule type="expression" dxfId="4" priority="33">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K2:K730">
-    <cfRule type="expression" dxfId="4" priority="5">
-      <formula>MOD(ROW(),2)=0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L3:P303 S256:T301 Q294:R303 S302:S303 T302:T305 L304:S305 A306:B489 Q306:R565 L306:P626 S306:T642 C306:C730 A493:B730 D653:H660 G659:I659 D661:F730">
+  <conditionalFormatting sqref="L3:P303 S256:T301 Q294:R303 S302:S303 T302:T305 L304:S305 A306:B489 Q306:R565 L306:P626 S306:T642 D653:H660 G659:I659">
     <cfRule type="expression" dxfId="3" priority="27">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L2:T2 Q3:T255 Q256:R287 Q566:Q628 R566:R642 M629:Q630 L631:Q642 L643:T650 M651:T652 R653:T693 L694:N730 Q694:T730">
+  <conditionalFormatting sqref="L2:T2 Q3:T255 Q256:R287 Q566:Q628 R566:R642 M629:Q630 L631:Q642 L643:T650 M651:T652 L685:N721 Q685:T721">
     <cfRule type="expression" dxfId="2" priority="44">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P653:Q685">
+  <conditionalFormatting sqref="P653:Q684">
     <cfRule type="expression" dxfId="1" priority="20">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q288:Q291 R288:R293 Q293 B490:B491 A490:A492 M627:P628 L627:L630 L651:L693 M653:O653 O653:O730 I654:I658 J654:J659 M654:N693 Q686:Q693 P686:P730">
+  <conditionalFormatting sqref="Q288:Q291 R288:R293 Q293 B490:B491 A490:A492 M627:P628 L627:L630 M653:O653 I654:I658 J654:J659">
     <cfRule type="expression" dxfId="0" priority="46">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>

</xml_diff>

<commit_message>
made some changes to answer key
</commit_message>
<xml_diff>
--- a/nvi_etl/survey/conf/nvi_answer_key_20260316.xlsx
+++ b/nvi_etl/survey/conf/nvi_answer_key_20260316.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\mike\2_responsibilities\nvi_etl\nvi_etl\survey\conf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E5B19DE-4816-4DEF-9047-43101A987B7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A26E532-8081-4DF7-B17E-3BF71F1028B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="18240" xr2:uid="{E6AADBC4-36D9-4E0B-9CAE-3CD032CDA67A}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" xr2:uid="{E6AADBC4-36D9-4E0B-9CAE-3CD032CDA67A}"/>
   </bookViews>
   <sheets>
     <sheet name="indicator_main" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6149" uniqueCount="742">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6149" uniqueCount="743">
   <si>
     <t>indicator_include</t>
   </si>
@@ -2020,9 +2020,6 @@
     <t>The condition of housing in your neighborhood</t>
   </si>
   <si>
-    <t>Do you have a family member who is or has been incarcerated in the last 12 months?</t>
-  </si>
-  <si>
     <t>Poor air quality</t>
   </si>
   <si>
@@ -2272,6 +2269,12 @@
   </si>
   <si>
     <t>Other (please describe)::Community_Engagement_Process_Participation...140</t>
+  </si>
+  <si>
+    <t>Do you have a family member who is or has been incarcerated in the last three years?</t>
+  </si>
+  <si>
+    <t>Youth_in_Household_Under5 == 1</t>
   </si>
 </sst>
 </file>
@@ -3346,7 +3349,7 @@
         <v>1</v>
       </c>
       <c r="E1" s="13" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>577</v>
@@ -3394,7 +3397,7 @@
         <v>11</v>
       </c>
       <c r="U1" s="15" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
     </row>
     <row r="2" spans="1:21" ht="20" x14ac:dyDescent="0.55000000000000004">
@@ -6397,7 +6400,7 @@
       </c>
       <c r="M49" s="2"/>
       <c r="N49" s="2" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="O49" s="2" t="s">
         <v>508</v>
@@ -6515,7 +6518,7 @@
       </c>
       <c r="M51" s="2"/>
       <c r="N51" s="2" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="O51" s="2" t="s">
         <v>508</v>
@@ -6574,7 +6577,7 @@
       </c>
       <c r="M52" s="2"/>
       <c r="N52" s="2" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="O52" s="2" t="s">
         <v>508</v>
@@ -14661,7 +14664,7 @@
         <v>590</v>
       </c>
       <c r="G182" s="2" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="H182" s="2" t="s">
         <v>36</v>
@@ -14724,7 +14727,7 @@
         <v>590</v>
       </c>
       <c r="G183" s="2" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="H183" s="2" t="s">
         <v>38</v>
@@ -14787,7 +14790,7 @@
         <v>590</v>
       </c>
       <c r="G184" s="2" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="H184" s="2" t="s">
         <v>39</v>
@@ -14850,7 +14853,7 @@
         <v>590</v>
       </c>
       <c r="G185" s="2" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="H185" s="2" t="s">
         <v>40</v>
@@ -14913,7 +14916,7 @@
         <v>590</v>
       </c>
       <c r="G186" s="2" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="H186" s="2" t="s">
         <v>41</v>
@@ -15901,7 +15904,7 @@
         <v>592</v>
       </c>
       <c r="G202" s="2" t="s">
-        <v>658</v>
+        <v>741</v>
       </c>
       <c r="H202" s="2" t="s">
         <v>122</v>
@@ -15938,7 +15941,7 @@
         <v>44927</v>
       </c>
       <c r="T202" s="14">
-        <v>45657</v>
+        <v>73050</v>
       </c>
       <c r="U202" s="16">
         <v>4</v>
@@ -15964,7 +15967,7 @@
         <v>592</v>
       </c>
       <c r="G203" s="2" t="s">
-        <v>658</v>
+        <v>741</v>
       </c>
       <c r="H203" s="2" t="s">
         <v>124</v>
@@ -16001,7 +16004,7 @@
         <v>44927</v>
       </c>
       <c r="T203" s="14">
-        <v>45657</v>
+        <v>73050</v>
       </c>
       <c r="U203" s="16">
         <v>4</v>
@@ -16027,7 +16030,7 @@
         <v>592</v>
       </c>
       <c r="G204" s="2" t="s">
-        <v>658</v>
+        <v>741</v>
       </c>
       <c r="H204" s="2" t="s">
         <v>125</v>
@@ -16064,7 +16067,7 @@
         <v>44927</v>
       </c>
       <c r="T204" s="14">
-        <v>45657</v>
+        <v>73050</v>
       </c>
       <c r="U204" s="16">
         <v>4</v>
@@ -16090,7 +16093,7 @@
         <v>593</v>
       </c>
       <c r="G205" s="2" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="H205" s="2" t="s">
         <v>362</v>
@@ -16153,7 +16156,7 @@
         <v>593</v>
       </c>
       <c r="G206" s="2" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="H206" s="2" t="s">
         <v>364</v>
@@ -16216,7 +16219,7 @@
         <v>593</v>
       </c>
       <c r="G207" s="2" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="H207" s="2" t="s">
         <v>365</v>
@@ -16279,7 +16282,7 @@
         <v>593</v>
       </c>
       <c r="G208" s="2" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="H208" s="2" t="s">
         <v>366</v>
@@ -16342,7 +16345,7 @@
         <v>593</v>
       </c>
       <c r="G209" s="2" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="H209" s="2" t="s">
         <v>367</v>
@@ -16405,7 +16408,7 @@
         <v>593</v>
       </c>
       <c r="G210" s="2" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="H210" s="2" t="s">
         <v>362</v>
@@ -16468,7 +16471,7 @@
         <v>593</v>
       </c>
       <c r="G211" s="2" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="H211" s="2" t="s">
         <v>364</v>
@@ -16531,7 +16534,7 @@
         <v>593</v>
       </c>
       <c r="G212" s="2" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="H212" s="2" t="s">
         <v>365</v>
@@ -16594,7 +16597,7 @@
         <v>593</v>
       </c>
       <c r="G213" s="2" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="H213" s="2" t="s">
         <v>366</v>
@@ -16657,7 +16660,7 @@
         <v>593</v>
       </c>
       <c r="G214" s="2" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="H214" s="2" t="s">
         <v>367</v>
@@ -17035,7 +17038,7 @@
         <v>593</v>
       </c>
       <c r="G220" s="2" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="H220" s="2" t="s">
         <v>362</v>
@@ -17098,7 +17101,7 @@
         <v>593</v>
       </c>
       <c r="G221" s="2" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="H221" s="2" t="s">
         <v>364</v>
@@ -17161,7 +17164,7 @@
         <v>593</v>
       </c>
       <c r="G222" s="2" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="H222" s="2" t="s">
         <v>365</v>
@@ -17224,7 +17227,7 @@
         <v>593</v>
       </c>
       <c r="G223" s="2" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="H223" s="2" t="s">
         <v>366</v>
@@ -17287,7 +17290,7 @@
         <v>593</v>
       </c>
       <c r="G224" s="2" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="H224" s="2" t="s">
         <v>367</v>
@@ -17350,7 +17353,7 @@
         <v>593</v>
       </c>
       <c r="G225" s="2" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="H225" s="2" t="s">
         <v>362</v>
@@ -17413,7 +17416,7 @@
         <v>593</v>
       </c>
       <c r="G226" s="2" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="H226" s="2" t="s">
         <v>364</v>
@@ -17476,7 +17479,7 @@
         <v>593</v>
       </c>
       <c r="G227" s="2" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="H227" s="2" t="s">
         <v>365</v>
@@ -17539,7 +17542,7 @@
         <v>593</v>
       </c>
       <c r="G228" s="2" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="H228" s="2" t="s">
         <v>366</v>
@@ -17602,7 +17605,7 @@
         <v>593</v>
       </c>
       <c r="G229" s="2" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="H229" s="2" t="s">
         <v>367</v>
@@ -17980,7 +17983,7 @@
         <v>593</v>
       </c>
       <c r="G235" s="2" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="H235" s="2" t="s">
         <v>362</v>
@@ -18043,7 +18046,7 @@
         <v>593</v>
       </c>
       <c r="G236" s="2" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="H236" s="2" t="s">
         <v>364</v>
@@ -18106,7 +18109,7 @@
         <v>593</v>
       </c>
       <c r="G237" s="2" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="H237" s="2" t="s">
         <v>365</v>
@@ -18169,7 +18172,7 @@
         <v>593</v>
       </c>
       <c r="G238" s="2" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="H238" s="2" t="s">
         <v>366</v>
@@ -18232,7 +18235,7 @@
         <v>593</v>
       </c>
       <c r="G239" s="2" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="H239" s="2" t="s">
         <v>367</v>
@@ -18295,7 +18298,7 @@
         <v>593</v>
       </c>
       <c r="G240" s="2" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="H240" s="2" t="s">
         <v>362</v>
@@ -18358,7 +18361,7 @@
         <v>593</v>
       </c>
       <c r="G241" s="2" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="H241" s="2" t="s">
         <v>364</v>
@@ -18421,7 +18424,7 @@
         <v>593</v>
       </c>
       <c r="G242" s="2" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="H242" s="2" t="s">
         <v>365</v>
@@ -18484,7 +18487,7 @@
         <v>593</v>
       </c>
       <c r="G243" s="2" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="H243" s="2" t="s">
         <v>366</v>
@@ -18547,7 +18550,7 @@
         <v>593</v>
       </c>
       <c r="G244" s="2" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="H244" s="2" t="s">
         <v>367</v>
@@ -18610,7 +18613,7 @@
         <v>593</v>
       </c>
       <c r="G245" s="2" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="H245" s="2" t="s">
         <v>362</v>
@@ -18673,7 +18676,7 @@
         <v>593</v>
       </c>
       <c r="G246" s="2" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="H246" s="2" t="s">
         <v>364</v>
@@ -18736,7 +18739,7 @@
         <v>593</v>
       </c>
       <c r="G247" s="2" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="H247" s="2" t="s">
         <v>365</v>
@@ -18799,7 +18802,7 @@
         <v>593</v>
       </c>
       <c r="G248" s="2" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="H248" s="2" t="s">
         <v>366</v>
@@ -18862,7 +18865,7 @@
         <v>593</v>
       </c>
       <c r="G249" s="2" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="H249" s="2" t="s">
         <v>367</v>
@@ -20167,7 +20170,7 @@
       </c>
       <c r="M271" s="2"/>
       <c r="N271" s="2" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="O271" s="2" t="s">
         <v>508</v>
@@ -20329,7 +20332,7 @@
         <v>598</v>
       </c>
       <c r="G274" s="2" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="H274" s="2" t="s">
         <v>122</v>
@@ -20392,7 +20395,7 @@
         <v>598</v>
       </c>
       <c r="G275" s="2" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="H275" s="2" t="s">
         <v>124</v>
@@ -20455,7 +20458,7 @@
         <v>598</v>
       </c>
       <c r="G276" s="2" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="H276" s="2" t="s">
         <v>125</v>
@@ -20533,7 +20536,7 @@
       </c>
       <c r="M277" s="2"/>
       <c r="N277" s="2" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="O277" s="2" t="s">
         <v>508</v>
@@ -20872,7 +20875,7 @@
         <v>592</v>
       </c>
       <c r="G283" s="2" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="H283" s="2" t="s">
         <v>122</v>
@@ -20935,7 +20938,7 @@
         <v>592</v>
       </c>
       <c r="G284" s="2" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="H284" s="2" t="s">
         <v>124</v>
@@ -20998,7 +21001,7 @@
         <v>592</v>
       </c>
       <c r="G285" s="2" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="H285" s="2" t="s">
         <v>125</v>
@@ -21194,7 +21197,7 @@
       </c>
       <c r="M288" s="2"/>
       <c r="N288" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="O288" s="2" t="s">
         <v>508</v>
@@ -22001,7 +22004,7 @@
       <c r="E302" s="2"/>
       <c r="F302" s="2"/>
       <c r="G302" s="2" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="H302" s="2" t="s">
         <v>122</v>
@@ -22020,7 +22023,7 @@
       </c>
       <c r="M302" s="2"/>
       <c r="N302" s="2" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="O302" s="2" t="s">
         <v>15</v>
@@ -22060,7 +22063,7 @@
       <c r="E303" s="2"/>
       <c r="F303" s="2"/>
       <c r="G303" s="2" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="H303" s="2" t="s">
         <v>124</v>
@@ -22079,7 +22082,7 @@
       </c>
       <c r="M303" s="2"/>
       <c r="N303" s="2" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="O303" s="2" t="s">
         <v>15</v>
@@ -22119,7 +22122,7 @@
       <c r="E304" s="2"/>
       <c r="F304" s="2"/>
       <c r="G304" s="2" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="H304" s="2" t="s">
         <v>122</v>
@@ -22138,7 +22141,7 @@
       </c>
       <c r="M304" s="2"/>
       <c r="N304" s="2" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="O304" s="2" t="s">
         <v>15</v>
@@ -22178,7 +22181,7 @@
       <c r="E305" s="2"/>
       <c r="F305" s="2"/>
       <c r="G305" s="2" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="H305" s="2" t="s">
         <v>124</v>
@@ -22197,7 +22200,7 @@
       </c>
       <c r="M305" s="2"/>
       <c r="N305" s="2" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="O305" s="2" t="s">
         <v>15</v>
@@ -22241,7 +22244,7 @@
         <v>602</v>
       </c>
       <c r="G306" s="2" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="H306" s="2" t="s">
         <v>384</v>
@@ -22304,7 +22307,7 @@
         <v>602</v>
       </c>
       <c r="G307" s="2" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="H307" s="2" t="s">
         <v>386</v>
@@ -22367,7 +22370,7 @@
         <v>602</v>
       </c>
       <c r="G308" s="2" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="H308" s="2" t="s">
         <v>387</v>
@@ -22430,7 +22433,7 @@
         <v>602</v>
       </c>
       <c r="G309" s="2" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="H309" s="2" t="s">
         <v>388</v>
@@ -22493,7 +22496,7 @@
         <v>602</v>
       </c>
       <c r="G310" s="2" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="H310" s="2" t="s">
         <v>529</v>
@@ -22867,7 +22870,7 @@
       <c r="E316" s="2"/>
       <c r="F316" s="2"/>
       <c r="G316" s="2" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="H316" s="2" t="s">
         <v>36</v>
@@ -22926,7 +22929,7 @@
       <c r="E317" s="2"/>
       <c r="F317" s="2"/>
       <c r="G317" s="2" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="H317" s="2" t="s">
         <v>38</v>
@@ -22985,7 +22988,7 @@
       <c r="E318" s="2"/>
       <c r="F318" s="2"/>
       <c r="G318" s="2" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="H318" s="2" t="s">
         <v>39</v>
@@ -23044,7 +23047,7 @@
       <c r="E319" s="2"/>
       <c r="F319" s="2"/>
       <c r="G319" s="2" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="H319" s="2" t="s">
         <v>40</v>
@@ -23103,7 +23106,7 @@
       <c r="E320" s="2"/>
       <c r="F320" s="2"/>
       <c r="G320" s="2" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="H320" s="2" t="s">
         <v>41</v>
@@ -23162,7 +23165,7 @@
       <c r="E321" s="2"/>
       <c r="F321" s="2"/>
       <c r="G321" s="2" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="H321" s="2" t="s">
         <v>125</v>
@@ -23225,7 +23228,7 @@
         <v>603</v>
       </c>
       <c r="G322" s="2" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="H322" s="2" t="s">
         <v>122</v>
@@ -23288,7 +23291,7 @@
         <v>603</v>
       </c>
       <c r="G323" s="2" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="H323" s="2" t="s">
         <v>124</v>
@@ -23636,7 +23639,7 @@
         <v>604</v>
       </c>
       <c r="G329" s="2" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="H329" s="2" t="s">
         <v>13</v>
@@ -23699,7 +23702,7 @@
         <v>604</v>
       </c>
       <c r="G330" s="2" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="H330" s="2" t="s">
         <v>16</v>
@@ -23762,7 +23765,7 @@
         <v>604</v>
       </c>
       <c r="G331" s="2" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="H331" s="2" t="s">
         <v>17</v>
@@ -23825,7 +23828,7 @@
         <v>604</v>
       </c>
       <c r="G332" s="2" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="H332" s="2" t="s">
         <v>13</v>
@@ -23888,7 +23891,7 @@
         <v>604</v>
       </c>
       <c r="G333" s="2" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="H333" s="2" t="s">
         <v>16</v>
@@ -23951,7 +23954,7 @@
         <v>604</v>
       </c>
       <c r="G334" s="2" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="H334" s="2" t="s">
         <v>17</v>
@@ -24014,7 +24017,7 @@
         <v>604</v>
       </c>
       <c r="G335" s="2" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="H335" s="2" t="s">
         <v>13</v>
@@ -24077,7 +24080,7 @@
         <v>604</v>
       </c>
       <c r="G336" s="2" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="H336" s="2" t="s">
         <v>16</v>
@@ -24140,7 +24143,7 @@
         <v>604</v>
       </c>
       <c r="G337" s="2" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="H337" s="2" t="s">
         <v>17</v>
@@ -24600,7 +24603,7 @@
         <v>578</v>
       </c>
       <c r="G345" s="2" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="H345" s="2" t="s">
         <v>36</v>
@@ -24663,7 +24666,7 @@
         <v>578</v>
       </c>
       <c r="G346" s="2" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="H346" s="2" t="s">
         <v>38</v>
@@ -24726,7 +24729,7 @@
         <v>578</v>
       </c>
       <c r="G347" s="2" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="H347" s="2" t="s">
         <v>39</v>
@@ -24789,7 +24792,7 @@
         <v>578</v>
       </c>
       <c r="G348" s="2" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="H348" s="2" t="s">
         <v>40</v>
@@ -24852,7 +24855,7 @@
         <v>578</v>
       </c>
       <c r="G349" s="2" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="H349" s="2" t="s">
         <v>41</v>
@@ -24915,7 +24918,7 @@
         <v>578</v>
       </c>
       <c r="G350" s="2" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="H350" s="2" t="s">
         <v>125</v>
@@ -24978,7 +24981,7 @@
         <v>578</v>
       </c>
       <c r="G351" s="2" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="H351" s="2" t="s">
         <v>36</v>
@@ -25041,7 +25044,7 @@
         <v>578</v>
       </c>
       <c r="G352" s="2" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="H352" s="2" t="s">
         <v>38</v>
@@ -25104,7 +25107,7 @@
         <v>578</v>
       </c>
       <c r="G353" s="2" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="H353" s="2" t="s">
         <v>39</v>
@@ -25167,7 +25170,7 @@
         <v>578</v>
       </c>
       <c r="G354" s="2" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="H354" s="2" t="s">
         <v>40</v>
@@ -25230,7 +25233,7 @@
         <v>578</v>
       </c>
       <c r="G355" s="2" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="H355" s="2" t="s">
         <v>41</v>
@@ -25293,7 +25296,7 @@
         <v>578</v>
       </c>
       <c r="G356" s="2" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="H356" s="2" t="s">
         <v>125</v>
@@ -25356,7 +25359,7 @@
         <v>605</v>
       </c>
       <c r="G357" s="2" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="H357" s="2" t="s">
         <v>21</v>
@@ -25419,7 +25422,7 @@
         <v>605</v>
       </c>
       <c r="G358" s="2" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="H358" s="2" t="s">
         <v>23</v>
@@ -25482,7 +25485,7 @@
         <v>605</v>
       </c>
       <c r="G359" s="2" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="H359" s="2" t="s">
         <v>24</v>
@@ -25545,7 +25548,7 @@
         <v>605</v>
       </c>
       <c r="G360" s="2" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="H360" s="2" t="s">
         <v>25</v>
@@ -25608,7 +25611,7 @@
         <v>605</v>
       </c>
       <c r="G361" s="2" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="H361" s="2" t="s">
         <v>21</v>
@@ -25671,7 +25674,7 @@
         <v>605</v>
       </c>
       <c r="G362" s="2" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="H362" s="2" t="s">
         <v>23</v>
@@ -25734,7 +25737,7 @@
         <v>605</v>
       </c>
       <c r="G363" s="2" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="H363" s="2" t="s">
         <v>24</v>
@@ -25797,7 +25800,7 @@
         <v>605</v>
       </c>
       <c r="G364" s="2" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="H364" s="2" t="s">
         <v>25</v>
@@ -25856,7 +25859,7 @@
       <c r="E365" s="2"/>
       <c r="F365" s="2"/>
       <c r="G365" s="2" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="H365" s="2" t="s">
         <v>55</v>
@@ -25915,7 +25918,7 @@
       <c r="E366" s="2"/>
       <c r="F366" s="2"/>
       <c r="G366" s="2" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="H366" s="2" t="s">
         <v>56</v>
@@ -25974,7 +25977,7 @@
       <c r="E367" s="2"/>
       <c r="F367" s="2"/>
       <c r="G367" s="2" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="H367" s="2" t="s">
         <v>57</v>
@@ -26033,7 +26036,7 @@
       <c r="E368" s="2"/>
       <c r="F368" s="2"/>
       <c r="G368" s="2" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="H368" s="2" t="s">
         <v>58</v>
@@ -26092,7 +26095,7 @@
       <c r="E369" s="2"/>
       <c r="F369" s="2"/>
       <c r="G369" s="2" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="H369" s="2" t="s">
         <v>59</v>
@@ -26308,7 +26311,7 @@
         <v>513</v>
       </c>
       <c r="R372" s="2" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="S372" s="9">
         <v>44927</v>
@@ -26367,7 +26370,7 @@
         <v>513</v>
       </c>
       <c r="R373" s="2" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="S373" s="9">
         <v>44927</v>
@@ -26426,7 +26429,7 @@
         <v>513</v>
       </c>
       <c r="R374" s="2" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="S374" s="9">
         <v>44927</v>
@@ -26485,7 +26488,7 @@
         <v>513</v>
       </c>
       <c r="R375" s="2" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="S375" s="9">
         <v>44927</v>
@@ -26544,7 +26547,7 @@
         <v>513</v>
       </c>
       <c r="R376" s="2" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="S376" s="9">
         <v>44927</v>
@@ -26603,7 +26606,7 @@
         <v>513</v>
       </c>
       <c r="R377" s="2" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="S377" s="9">
         <v>44927</v>
@@ -26662,7 +26665,7 @@
         <v>513</v>
       </c>
       <c r="R378" s="2" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="S378" s="9">
         <v>44927</v>
@@ -26721,7 +26724,7 @@
         <v>513</v>
       </c>
       <c r="R379" s="2" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="S379" s="9">
         <v>44927</v>
@@ -26780,7 +26783,7 @@
         <v>513</v>
       </c>
       <c r="R380" s="2" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="S380" s="9">
         <v>44927</v>
@@ -26839,7 +26842,7 @@
         <v>513</v>
       </c>
       <c r="R381" s="2" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="S381" s="9">
         <v>44927</v>
@@ -26898,7 +26901,7 @@
         <v>513</v>
       </c>
       <c r="R382" s="2" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="S382" s="9">
         <v>44927</v>
@@ -26957,7 +26960,7 @@
         <v>513</v>
       </c>
       <c r="R383" s="2" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="S383" s="9">
         <v>44927</v>
@@ -27016,7 +27019,7 @@
         <v>513</v>
       </c>
       <c r="R384" s="2" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="S384" s="9">
         <v>44927</v>
@@ -27046,7 +27049,7 @@
         <v>590</v>
       </c>
       <c r="G385" s="2" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="H385" s="2" t="s">
         <v>36</v>
@@ -27107,7 +27110,7 @@
         <v>590</v>
       </c>
       <c r="G386" s="2" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="H386" s="2" t="s">
         <v>38</v>
@@ -27168,7 +27171,7 @@
         <v>590</v>
       </c>
       <c r="G387" s="2" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="H387" s="2" t="s">
         <v>39</v>
@@ -27229,7 +27232,7 @@
         <v>590</v>
       </c>
       <c r="G388" s="2" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="H388" s="2" t="s">
         <v>40</v>
@@ -27290,7 +27293,7 @@
         <v>590</v>
       </c>
       <c r="G389" s="2" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="H389" s="2" t="s">
         <v>41</v>
@@ -27353,7 +27356,7 @@
         <v>590</v>
       </c>
       <c r="G390" s="2" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="H390" s="2" t="s">
         <v>36</v>
@@ -27416,7 +27419,7 @@
         <v>590</v>
       </c>
       <c r="G391" s="2" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="H391" s="2" t="s">
         <v>38</v>
@@ -27479,7 +27482,7 @@
         <v>590</v>
       </c>
       <c r="G392" s="2" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="H392" s="2" t="s">
         <v>39</v>
@@ -27542,7 +27545,7 @@
         <v>590</v>
       </c>
       <c r="G393" s="2" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="H393" s="2" t="s">
         <v>40</v>
@@ -27605,7 +27608,7 @@
         <v>590</v>
       </c>
       <c r="G394" s="2" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="H394" s="2" t="s">
         <v>41</v>
@@ -27668,7 +27671,7 @@
         <v>590</v>
       </c>
       <c r="G395" s="2" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="H395" s="2" t="s">
         <v>36</v>
@@ -27731,7 +27734,7 @@
         <v>590</v>
       </c>
       <c r="G396" s="2" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="H396" s="2" t="s">
         <v>38</v>
@@ -27794,7 +27797,7 @@
         <v>590</v>
       </c>
       <c r="G397" s="2" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="H397" s="2" t="s">
         <v>39</v>
@@ -27857,7 +27860,7 @@
         <v>590</v>
       </c>
       <c r="G398" s="2" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="H398" s="2" t="s">
         <v>40</v>
@@ -27920,7 +27923,7 @@
         <v>590</v>
       </c>
       <c r="G399" s="2" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="H399" s="2" t="s">
         <v>41</v>
@@ -27981,7 +27984,7 @@
         <v>590</v>
       </c>
       <c r="G400" s="2" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="H400" s="2" t="s">
         <v>36</v>
@@ -28042,7 +28045,7 @@
         <v>590</v>
       </c>
       <c r="G401" s="2" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="H401" s="2" t="s">
         <v>38</v>
@@ -28103,7 +28106,7 @@
         <v>590</v>
       </c>
       <c r="G402" s="2" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="H402" s="2" t="s">
         <v>39</v>
@@ -28164,7 +28167,7 @@
         <v>590</v>
       </c>
       <c r="G403" s="2" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="H403" s="2" t="s">
         <v>40</v>
@@ -28225,7 +28228,7 @@
         <v>590</v>
       </c>
       <c r="G404" s="2" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="H404" s="2" t="s">
         <v>41</v>
@@ -28671,7 +28674,7 @@
       </c>
       <c r="M411" s="2"/>
       <c r="N411" s="2" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="O411" s="2" t="s">
         <v>508</v>
@@ -28732,7 +28735,7 @@
       </c>
       <c r="M412" s="2"/>
       <c r="N412" s="2" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="O412" s="2" t="s">
         <v>508</v>
@@ -28793,7 +28796,7 @@
       </c>
       <c r="M413" s="2"/>
       <c r="N413" s="2" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="O413" s="2" t="s">
         <v>508</v>
@@ -28854,7 +28857,7 @@
       </c>
       <c r="M414" s="2"/>
       <c r="N414" s="2" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="O414" s="2" t="s">
         <v>508</v>
@@ -28915,7 +28918,7 @@
       </c>
       <c r="M415" s="2"/>
       <c r="N415" s="2" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="O415" s="2" t="s">
         <v>508</v>
@@ -28976,7 +28979,7 @@
       </c>
       <c r="M416" s="2"/>
       <c r="N416" s="2" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="O416" s="2" t="s">
         <v>508</v>
@@ -29769,7 +29772,7 @@
       </c>
       <c r="M429" s="2"/>
       <c r="N429" s="2" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="O429" s="2" t="s">
         <v>508</v>
@@ -29830,7 +29833,7 @@
       </c>
       <c r="M430" s="2"/>
       <c r="N430" s="2" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="O430" s="2" t="s">
         <v>508</v>
@@ -29891,7 +29894,7 @@
       </c>
       <c r="M431" s="2"/>
       <c r="N431" s="2" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="O431" s="2" t="s">
         <v>508</v>
@@ -29952,7 +29955,7 @@
       </c>
       <c r="M432" s="2"/>
       <c r="N432" s="2" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="O432" s="2" t="s">
         <v>508</v>
@@ -30013,7 +30016,7 @@
       </c>
       <c r="M433" s="2"/>
       <c r="N433" s="2" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="O433" s="2" t="s">
         <v>508</v>
@@ -30074,7 +30077,7 @@
       </c>
       <c r="M434" s="2"/>
       <c r="N434" s="2" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="O434" s="2" t="s">
         <v>508</v>
@@ -32672,7 +32675,7 @@
       <c r="E479" s="2"/>
       <c r="F479" s="2"/>
       <c r="G479" s="2" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="H479" s="2" t="s">
         <v>245</v>
@@ -32727,7 +32730,7 @@
       <c r="E480" s="2"/>
       <c r="F480" s="2"/>
       <c r="G480" s="2" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="H480" s="2" t="s">
         <v>247</v>
@@ -32782,7 +32785,7 @@
       <c r="E481" s="2"/>
       <c r="F481" s="2"/>
       <c r="G481" s="2" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="H481" s="2" t="s">
         <v>249</v>
@@ -32837,7 +32840,7 @@
       <c r="E482" s="2"/>
       <c r="F482" s="2"/>
       <c r="G482" s="2" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="H482" s="2" t="s">
         <v>251</v>
@@ -32892,7 +32895,7 @@
       <c r="E483" s="2"/>
       <c r="F483" s="2"/>
       <c r="G483" s="2" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="H483" s="2" t="s">
         <v>253</v>
@@ -32947,7 +32950,7 @@
       <c r="E484" s="2"/>
       <c r="F484" s="2"/>
       <c r="G484" s="2" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="H484" s="2" t="s">
         <v>255</v>
@@ -33002,7 +33005,7 @@
       <c r="E485" s="2"/>
       <c r="F485" s="2"/>
       <c r="G485" s="2" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="H485" s="2" t="s">
         <v>257</v>
@@ -33973,7 +33976,7 @@
         <v>612</v>
       </c>
       <c r="G502" s="2" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="H502" s="2" t="s">
         <v>287</v>
@@ -34034,7 +34037,7 @@
         <v>612</v>
       </c>
       <c r="G503" s="2" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="H503" s="2" t="s">
         <v>289</v>
@@ -34095,7 +34098,7 @@
         <v>612</v>
       </c>
       <c r="G504" s="2" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="H504" s="2" t="s">
         <v>290</v>
@@ -34156,7 +34159,7 @@
         <v>612</v>
       </c>
       <c r="G505" s="2" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="H505" s="2" t="s">
         <v>291</v>
@@ -34217,7 +34220,7 @@
         <v>612</v>
       </c>
       <c r="G506" s="2" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="H506" s="2" t="s">
         <v>292</v>
@@ -34278,7 +34281,7 @@
         <v>612</v>
       </c>
       <c r="G507" s="2" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="H507" s="2" t="s">
         <v>287</v>
@@ -34339,7 +34342,7 @@
         <v>612</v>
       </c>
       <c r="G508" s="2" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="H508" s="2" t="s">
         <v>289</v>
@@ -34400,7 +34403,7 @@
         <v>612</v>
       </c>
       <c r="G509" s="2" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="H509" s="2" t="s">
         <v>290</v>
@@ -34461,7 +34464,7 @@
         <v>612</v>
       </c>
       <c r="G510" s="2" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="H510" s="2" t="s">
         <v>291</v>
@@ -34522,7 +34525,7 @@
         <v>612</v>
       </c>
       <c r="G511" s="2" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="H511" s="2" t="s">
         <v>292</v>
@@ -34583,7 +34586,7 @@
         <v>612</v>
       </c>
       <c r="G512" s="2" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="H512" s="2" t="s">
         <v>287</v>
@@ -34644,7 +34647,7 @@
         <v>612</v>
       </c>
       <c r="G513" s="2" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="H513" s="2" t="s">
         <v>289</v>
@@ -34705,7 +34708,7 @@
         <v>612</v>
       </c>
       <c r="G514" s="2" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="H514" s="2" t="s">
         <v>290</v>
@@ -34766,7 +34769,7 @@
         <v>612</v>
       </c>
       <c r="G515" s="2" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="H515" s="2" t="s">
         <v>291</v>
@@ -34827,7 +34830,7 @@
         <v>612</v>
       </c>
       <c r="G516" s="2" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="H516" s="2" t="s">
         <v>292</v>
@@ -34888,7 +34891,7 @@
         <v>612</v>
       </c>
       <c r="G517" s="2" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="H517" s="2" t="s">
         <v>287</v>
@@ -34949,7 +34952,7 @@
         <v>612</v>
       </c>
       <c r="G518" s="2" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="H518" s="2" t="s">
         <v>289</v>
@@ -35010,7 +35013,7 @@
         <v>612</v>
       </c>
       <c r="G519" s="2" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="H519" s="2" t="s">
         <v>290</v>
@@ -35071,7 +35074,7 @@
         <v>612</v>
       </c>
       <c r="G520" s="2" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="H520" s="2" t="s">
         <v>291</v>
@@ -35132,7 +35135,7 @@
         <v>612</v>
       </c>
       <c r="G521" s="2" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="H521" s="2" t="s">
         <v>292</v>
@@ -35193,7 +35196,7 @@
         <v>612</v>
       </c>
       <c r="G522" s="2" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="H522" s="2" t="s">
         <v>287</v>
@@ -35254,7 +35257,7 @@
         <v>612</v>
       </c>
       <c r="G523" s="2" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="H523" s="2" t="s">
         <v>289</v>
@@ -35315,7 +35318,7 @@
         <v>612</v>
       </c>
       <c r="G524" s="2" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="H524" s="2" t="s">
         <v>290</v>
@@ -35376,7 +35379,7 @@
         <v>612</v>
       </c>
       <c r="G525" s="2" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="H525" s="2" t="s">
         <v>291</v>
@@ -35437,7 +35440,7 @@
         <v>612</v>
       </c>
       <c r="G526" s="2" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="H526" s="2" t="s">
         <v>292</v>
@@ -35498,7 +35501,7 @@
         <v>612</v>
       </c>
       <c r="G527" s="2" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="H527" s="2" t="s">
         <v>287</v>
@@ -35559,7 +35562,7 @@
         <v>612</v>
       </c>
       <c r="G528" s="2" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="H528" s="2" t="s">
         <v>289</v>
@@ -35620,7 +35623,7 @@
         <v>612</v>
       </c>
       <c r="G529" s="2" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="H529" s="2" t="s">
         <v>290</v>
@@ -35681,7 +35684,7 @@
         <v>612</v>
       </c>
       <c r="G530" s="2" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="H530" s="2" t="s">
         <v>291</v>
@@ -35742,7 +35745,7 @@
         <v>612</v>
       </c>
       <c r="G531" s="2" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="H531" s="2" t="s">
         <v>292</v>
@@ -35803,7 +35806,7 @@
         <v>612</v>
       </c>
       <c r="G532" s="2" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="H532" s="2" t="s">
         <v>287</v>
@@ -35864,7 +35867,7 @@
         <v>612</v>
       </c>
       <c r="G533" s="2" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="H533" s="2" t="s">
         <v>289</v>
@@ -35925,7 +35928,7 @@
         <v>612</v>
       </c>
       <c r="G534" s="2" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="H534" s="2" t="s">
         <v>290</v>
@@ -35986,7 +35989,7 @@
         <v>612</v>
       </c>
       <c r="G535" s="2" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="H535" s="2" t="s">
         <v>291</v>
@@ -36047,7 +36050,7 @@
         <v>612</v>
       </c>
       <c r="G536" s="2" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="H536" s="2" t="s">
         <v>292</v>
@@ -36108,7 +36111,7 @@
         <v>612</v>
       </c>
       <c r="G537" s="2" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="H537" s="2" t="s">
         <v>287</v>
@@ -36169,7 +36172,7 @@
         <v>612</v>
       </c>
       <c r="G538" s="2" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="H538" s="2" t="s">
         <v>289</v>
@@ -36230,7 +36233,7 @@
         <v>612</v>
       </c>
       <c r="G539" s="2" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="H539" s="2" t="s">
         <v>290</v>
@@ -36291,7 +36294,7 @@
         <v>612</v>
       </c>
       <c r="G540" s="2" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="H540" s="2" t="s">
         <v>291</v>
@@ -36352,7 +36355,7 @@
         <v>612</v>
       </c>
       <c r="G541" s="2" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="H541" s="2" t="s">
         <v>292</v>
@@ -36413,7 +36416,7 @@
         <v>612</v>
       </c>
       <c r="G542" s="2" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="H542" s="2" t="s">
         <v>287</v>
@@ -36474,7 +36477,7 @@
         <v>612</v>
       </c>
       <c r="G543" s="2" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="H543" s="2" t="s">
         <v>289</v>
@@ -36535,7 +36538,7 @@
         <v>612</v>
       </c>
       <c r="G544" s="2" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="H544" s="2" t="s">
         <v>290</v>
@@ -36596,7 +36599,7 @@
         <v>612</v>
       </c>
       <c r="G545" s="2" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="H545" s="2" t="s">
         <v>291</v>
@@ -36657,7 +36660,7 @@
         <v>612</v>
       </c>
       <c r="G546" s="2" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="H546" s="2" t="s">
         <v>292</v>
@@ -36718,7 +36721,7 @@
         <v>612</v>
       </c>
       <c r="G547" s="2" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="H547" s="2" t="s">
         <v>287</v>
@@ -36779,7 +36782,7 @@
         <v>612</v>
       </c>
       <c r="G548" s="2" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="H548" s="2" t="s">
         <v>289</v>
@@ -36840,7 +36843,7 @@
         <v>612</v>
       </c>
       <c r="G549" s="2" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="H549" s="2" t="s">
         <v>290</v>
@@ -36901,7 +36904,7 @@
         <v>612</v>
       </c>
       <c r="G550" s="2" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="H550" s="2" t="s">
         <v>291</v>
@@ -36962,7 +36965,7 @@
         <v>612</v>
       </c>
       <c r="G551" s="2" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="H551" s="2" t="s">
         <v>292</v>
@@ -37023,7 +37026,7 @@
         <v>612</v>
       </c>
       <c r="G552" s="2" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="H552" s="2" t="s">
         <v>287</v>
@@ -37084,7 +37087,7 @@
         <v>612</v>
       </c>
       <c r="G553" s="2" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="H553" s="2" t="s">
         <v>289</v>
@@ -37145,7 +37148,7 @@
         <v>612</v>
       </c>
       <c r="G554" s="2" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="H554" s="2" t="s">
         <v>290</v>
@@ -37206,7 +37209,7 @@
         <v>612</v>
       </c>
       <c r="G555" s="2" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="H555" s="2" t="s">
         <v>291</v>
@@ -37267,7 +37270,7 @@
         <v>612</v>
       </c>
       <c r="G556" s="2" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="H556" s="2" t="s">
         <v>292</v>
@@ -37477,7 +37480,7 @@
         <v>591</v>
       </c>
       <c r="G560" s="2" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="H560" s="2" t="s">
         <v>125</v>
@@ -37540,7 +37543,7 @@
         <v>591</v>
       </c>
       <c r="G561" s="2" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="H561" s="2" t="s">
         <v>122</v>
@@ -37603,7 +37606,7 @@
         <v>591</v>
       </c>
       <c r="G562" s="2" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="H562" s="2" t="s">
         <v>124</v>
@@ -37664,7 +37667,7 @@
         <v>591</v>
       </c>
       <c r="G563" s="2" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="H563" s="2" t="s">
         <v>125</v>
@@ -37725,7 +37728,7 @@
         <v>591</v>
       </c>
       <c r="G564" s="2" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="H564" s="2" t="s">
         <v>122</v>
@@ -37786,7 +37789,7 @@
         <v>591</v>
       </c>
       <c r="G565" s="2" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="H565" s="2" t="s">
         <v>124</v>
@@ -38038,7 +38041,7 @@
         <v>598</v>
       </c>
       <c r="G569" s="2" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="H569" s="2" t="s">
         <v>122</v>
@@ -38101,7 +38104,7 @@
         <v>598</v>
       </c>
       <c r="G570" s="2" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="H570" s="2" t="s">
         <v>124</v>
@@ -38164,7 +38167,7 @@
         <v>598</v>
       </c>
       <c r="G571" s="2" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="H571" s="2" t="s">
         <v>125</v>
@@ -38461,7 +38464,7 @@
       <c r="E576" s="2"/>
       <c r="F576" s="2"/>
       <c r="G576" s="2" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="H576" s="2" t="s">
         <v>404</v>
@@ -38520,7 +38523,7 @@
       <c r="E577" s="2"/>
       <c r="F577" s="2"/>
       <c r="G577" s="2" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="H577" s="2" t="s">
         <v>405</v>
@@ -38579,7 +38582,7 @@
       <c r="E578" s="2"/>
       <c r="F578" s="2"/>
       <c r="G578" s="2" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="H578" s="2" t="s">
         <v>406</v>
@@ -38638,7 +38641,7 @@
       <c r="E579" s="2"/>
       <c r="F579" s="2"/>
       <c r="G579" s="2" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="H579" s="2" t="s">
         <v>407</v>
@@ -38697,7 +38700,7 @@
       <c r="E580" s="2"/>
       <c r="F580" s="2"/>
       <c r="G580" s="2" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="H580" s="2" t="s">
         <v>408</v>
@@ -38756,7 +38759,7 @@
       <c r="E581" s="2"/>
       <c r="F581" s="2"/>
       <c r="G581" s="2" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="H581" s="2" t="s">
         <v>409</v>
@@ -38815,7 +38818,7 @@
       <c r="E582" s="2"/>
       <c r="F582" s="2"/>
       <c r="G582" s="2" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="H582" s="2" t="s">
         <v>410</v>
@@ -38874,7 +38877,7 @@
       <c r="E583" s="2"/>
       <c r="F583" s="2"/>
       <c r="G583" s="2" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="H583" s="2" t="s">
         <v>411</v>
@@ -38933,7 +38936,7 @@
       <c r="E584" s="2"/>
       <c r="F584" s="2"/>
       <c r="G584" s="2" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="H584" s="2" t="s">
         <v>412</v>
@@ -39416,7 +39419,7 @@
       </c>
       <c r="M592" s="2"/>
       <c r="N592" s="2" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="O592" s="2" t="s">
         <v>508</v>
@@ -40680,7 +40683,7 @@
         <v>584</v>
       </c>
       <c r="G615" s="2" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="H615" s="2" t="s">
         <v>462</v>
@@ -40743,7 +40746,7 @@
         <v>584</v>
       </c>
       <c r="G616" s="2" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="H616" s="2" t="s">
         <v>464</v>
@@ -40806,7 +40809,7 @@
         <v>584</v>
       </c>
       <c r="G617" s="2" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="H617" s="2" t="s">
         <v>465</v>
@@ -40869,7 +40872,7 @@
         <v>584</v>
       </c>
       <c r="G618" s="2" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="H618" s="2" t="s">
         <v>466</v>
@@ -40932,7 +40935,7 @@
         <v>584</v>
       </c>
       <c r="G619" s="2" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="H619" s="2" t="s">
         <v>467</v>
@@ -42180,7 +42183,7 @@
       <c r="E641" s="2"/>
       <c r="F641" s="2"/>
       <c r="G641" s="2" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="H641" s="2" t="s">
         <v>122</v>
@@ -42237,7 +42240,7 @@
       <c r="E642" s="2"/>
       <c r="F642" s="2"/>
       <c r="G642" s="2" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="H642" s="2" t="s">
         <v>124</v>
@@ -42296,7 +42299,7 @@
       <c r="E643" s="2"/>
       <c r="F643" s="2"/>
       <c r="G643" s="2" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="H643" s="2" t="s">
         <v>207</v>
@@ -42355,7 +42358,7 @@
       <c r="E644" s="2"/>
       <c r="F644" s="2"/>
       <c r="G644" s="2" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="H644" s="2" t="s">
         <v>208</v>
@@ -42414,7 +42417,7 @@
       <c r="E645" s="2"/>
       <c r="F645" s="2"/>
       <c r="G645" s="2" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="H645" s="2" t="s">
         <v>527</v>
@@ -42473,7 +42476,7 @@
       <c r="E646" s="2"/>
       <c r="F646" s="2"/>
       <c r="G646" s="2" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="H646" s="2" t="s">
         <v>209</v>
@@ -42532,7 +42535,7 @@
       <c r="E647" s="2"/>
       <c r="F647" s="2"/>
       <c r="G647" s="2" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="H647" s="2" t="s">
         <v>210</v>
@@ -42591,7 +42594,7 @@
       <c r="E648" s="2"/>
       <c r="F648" s="2"/>
       <c r="G648" s="2" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="H648" s="2" t="s">
         <v>211</v>
@@ -42648,7 +42651,7 @@
       <c r="E649" s="2"/>
       <c r="F649" s="2"/>
       <c r="G649" s="2" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="H649" s="7" t="s">
         <v>124</v>
@@ -42703,7 +42706,7 @@
       <c r="E650" s="2"/>
       <c r="F650" s="2"/>
       <c r="G650" s="2" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="H650" s="7" t="s">
         <v>122</v>
@@ -42760,7 +42763,7 @@
       <c r="E651" s="2"/>
       <c r="F651" s="2"/>
       <c r="G651" s="2" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="H651" s="7" t="s">
         <v>124</v>
@@ -42817,7 +42820,7 @@
       <c r="E652" s="2"/>
       <c r="F652" s="2"/>
       <c r="G652" s="2" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="H652" s="7" t="s">
         <v>122</v>
@@ -42899,7 +42902,7 @@
         <v>508</v>
       </c>
       <c r="P653" s="2" t="s">
-        <v>520</v>
+        <v>742</v>
       </c>
       <c r="Q653" s="2"/>
       <c r="R653" s="2" t="s">
@@ -42956,7 +42959,7 @@
         <v>508</v>
       </c>
       <c r="P654" s="2" t="s">
-        <v>520</v>
+        <v>742</v>
       </c>
       <c r="Q654" s="2"/>
       <c r="R654" s="2" t="s">
@@ -43013,7 +43016,7 @@
         <v>508</v>
       </c>
       <c r="P655" s="2" t="s">
-        <v>520</v>
+        <v>742</v>
       </c>
       <c r="Q655" s="2"/>
       <c r="R655" s="2" t="s">
@@ -43070,7 +43073,7 @@
         <v>508</v>
       </c>
       <c r="P656" s="2" t="s">
-        <v>520</v>
+        <v>742</v>
       </c>
       <c r="Q656" s="2"/>
       <c r="R656" s="2" t="s">
@@ -43127,7 +43130,7 @@
         <v>508</v>
       </c>
       <c r="P657" s="2" t="s">
-        <v>520</v>
+        <v>742</v>
       </c>
       <c r="Q657" s="2"/>
       <c r="R657" s="2" t="s">
@@ -43184,7 +43187,7 @@
         <v>508</v>
       </c>
       <c r="P658" s="2" t="s">
-        <v>520</v>
+        <v>742</v>
       </c>
       <c r="Q658" s="2"/>
       <c r="R658" s="2" t="s">
@@ -43241,7 +43244,7 @@
         <v>508</v>
       </c>
       <c r="P659" s="2" t="s">
-        <v>520</v>
+        <v>742</v>
       </c>
       <c r="Q659" s="2"/>
       <c r="R659" s="2" t="s">
@@ -43277,7 +43280,7 @@
         <v>620</v>
       </c>
       <c r="G660" s="2" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="H660" s="2" t="s">
         <v>547</v>
@@ -43338,7 +43341,7 @@
         <v>620</v>
       </c>
       <c r="G661" s="2" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="H661" s="2" t="s">
         <v>546</v>
@@ -43399,7 +43402,7 @@
         <v>620</v>
       </c>
       <c r="G662" s="2" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="H662" s="2" t="s">
         <v>545</v>
@@ -43460,7 +43463,7 @@
         <v>620</v>
       </c>
       <c r="G663" s="2" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="H663" s="2" t="s">
         <v>544</v>
@@ -43521,7 +43524,7 @@
         <v>620</v>
       </c>
       <c r="G664" s="2" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="H664" s="2" t="s">
         <v>543</v>
@@ -43582,7 +43585,7 @@
         <v>620</v>
       </c>
       <c r="G665" s="2" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="H665" s="2" t="s">
         <v>547</v>
@@ -43643,7 +43646,7 @@
         <v>620</v>
       </c>
       <c r="G666" s="2" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="H666" s="2" t="s">
         <v>546</v>
@@ -43704,7 +43707,7 @@
         <v>620</v>
       </c>
       <c r="G667" s="2" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="H667" s="2" t="s">
         <v>545</v>
@@ -43765,7 +43768,7 @@
         <v>620</v>
       </c>
       <c r="G668" s="2" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="H668" s="2" t="s">
         <v>544</v>
@@ -43826,7 +43829,7 @@
         <v>620</v>
       </c>
       <c r="G669" s="2" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="H669" s="2" t="s">
         <v>543</v>
@@ -43887,7 +43890,7 @@
         <v>620</v>
       </c>
       <c r="G670" s="2" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="H670" s="2" t="s">
         <v>547</v>
@@ -43948,7 +43951,7 @@
         <v>620</v>
       </c>
       <c r="G671" s="2" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="H671" s="2" t="s">
         <v>546</v>
@@ -44009,7 +44012,7 @@
         <v>620</v>
       </c>
       <c r="G672" s="2" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="H672" s="2" t="s">
         <v>545</v>
@@ -44070,7 +44073,7 @@
         <v>620</v>
       </c>
       <c r="G673" s="2" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="H673" s="2" t="s">
         <v>544</v>
@@ -44131,7 +44134,7 @@
         <v>620</v>
       </c>
       <c r="G674" s="2" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="H674" s="2" t="s">
         <v>543</v>
@@ -44192,7 +44195,7 @@
         <v>620</v>
       </c>
       <c r="G675" s="2" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="H675" s="2" t="s">
         <v>547</v>
@@ -44253,7 +44256,7 @@
         <v>620</v>
       </c>
       <c r="G676" s="2" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="H676" s="2" t="s">
         <v>546</v>
@@ -44314,7 +44317,7 @@
         <v>620</v>
       </c>
       <c r="G677" s="2" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="H677" s="2" t="s">
         <v>545</v>
@@ -44375,7 +44378,7 @@
         <v>620</v>
       </c>
       <c r="G678" s="2" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="H678" s="2" t="s">
         <v>544</v>
@@ -44436,7 +44439,7 @@
         <v>620</v>
       </c>
       <c r="G679" s="2" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="H679" s="2" t="s">
         <v>543</v>
@@ -44497,7 +44500,7 @@
         <v>620</v>
       </c>
       <c r="G680" s="2" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="H680" s="2" t="s">
         <v>547</v>
@@ -44558,7 +44561,7 @@
         <v>620</v>
       </c>
       <c r="G681" s="2" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="H681" s="2" t="s">
         <v>546</v>
@@ -44619,7 +44622,7 @@
         <v>620</v>
       </c>
       <c r="G682" s="2" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="H682" s="2" t="s">
         <v>545</v>
@@ -44680,7 +44683,7 @@
         <v>620</v>
       </c>
       <c r="G683" s="2" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="H683" s="2" t="s">
         <v>544</v>
@@ -44741,7 +44744,7 @@
         <v>620</v>
       </c>
       <c r="G684" s="2" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="H684" s="2" t="s">
         <v>543</v>
@@ -44800,7 +44803,7 @@
         <v>621</v>
       </c>
       <c r="G685" s="2" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="H685" s="2" t="s">
         <v>549</v>
@@ -44859,7 +44862,7 @@
         <v>621</v>
       </c>
       <c r="G686" s="2" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="H686" s="2" t="s">
         <v>287</v>
@@ -44918,7 +44921,7 @@
         <v>621</v>
       </c>
       <c r="G687" s="2" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="H687" s="2" t="s">
         <v>289</v>
@@ -44977,7 +44980,7 @@
         <v>621</v>
       </c>
       <c r="G688" s="2" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="H688" s="2" t="s">
         <v>550</v>
@@ -45036,7 +45039,7 @@
         <v>621</v>
       </c>
       <c r="G689" s="2" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="H689" s="2" t="s">
         <v>551</v>
@@ -45095,7 +45098,7 @@
         <v>621</v>
       </c>
       <c r="G690" s="2" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="H690" s="2" t="s">
         <v>549</v>
@@ -45154,7 +45157,7 @@
         <v>621</v>
       </c>
       <c r="G691" s="2" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="H691" s="2" t="s">
         <v>287</v>
@@ -45213,7 +45216,7 @@
         <v>621</v>
       </c>
       <c r="G692" s="2" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="H692" s="2" t="s">
         <v>289</v>
@@ -45272,7 +45275,7 @@
         <v>621</v>
       </c>
       <c r="G693" s="2" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="H693" s="2" t="s">
         <v>550</v>
@@ -45331,7 +45334,7 @@
         <v>621</v>
       </c>
       <c r="G694" s="2" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="H694" s="2" t="s">
         <v>551</v>
@@ -45390,7 +45393,7 @@
         <v>621</v>
       </c>
       <c r="G695" s="2" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="H695" s="2" t="s">
         <v>549</v>
@@ -45449,7 +45452,7 @@
         <v>621</v>
       </c>
       <c r="G696" s="2" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="H696" s="2" t="s">
         <v>287</v>
@@ -45508,7 +45511,7 @@
         <v>621</v>
       </c>
       <c r="G697" s="2" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="H697" s="2" t="s">
         <v>289</v>
@@ -45567,7 +45570,7 @@
         <v>621</v>
       </c>
       <c r="G698" s="2" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="H698" s="2" t="s">
         <v>550</v>
@@ -45626,7 +45629,7 @@
         <v>621</v>
       </c>
       <c r="G699" s="2" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="H699" s="2" t="s">
         <v>551</v>
@@ -45685,7 +45688,7 @@
         <v>621</v>
       </c>
       <c r="G700" s="2" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="H700" s="2" t="s">
         <v>549</v>
@@ -45744,7 +45747,7 @@
         <v>621</v>
       </c>
       <c r="G701" s="2" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="H701" s="2" t="s">
         <v>287</v>
@@ -45803,7 +45806,7 @@
         <v>621</v>
       </c>
       <c r="G702" s="2" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="H702" s="2" t="s">
         <v>289</v>
@@ -45862,7 +45865,7 @@
         <v>621</v>
       </c>
       <c r="G703" s="2" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="H703" s="2" t="s">
         <v>550</v>
@@ -45921,7 +45924,7 @@
         <v>621</v>
       </c>
       <c r="G704" s="2" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="H704" s="2" t="s">
         <v>551</v>
@@ -45980,7 +45983,7 @@
         <v>621</v>
       </c>
       <c r="G705" s="2" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="H705" s="2" t="s">
         <v>549</v>
@@ -46039,7 +46042,7 @@
         <v>621</v>
       </c>
       <c r="G706" s="2" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="H706" s="2" t="s">
         <v>287</v>
@@ -46098,7 +46101,7 @@
         <v>621</v>
       </c>
       <c r="G707" s="2" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="H707" s="2" t="s">
         <v>289</v>
@@ -46157,7 +46160,7 @@
         <v>621</v>
       </c>
       <c r="G708" s="2" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="H708" s="2" t="s">
         <v>550</v>
@@ -46216,7 +46219,7 @@
         <v>621</v>
       </c>
       <c r="G709" s="2" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="H709" s="2" t="s">
         <v>551</v>
@@ -46275,7 +46278,7 @@
         <v>622</v>
       </c>
       <c r="G710" s="2" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="H710" s="2" t="s">
         <v>528</v>
@@ -46334,7 +46337,7 @@
         <v>622</v>
       </c>
       <c r="G711" s="2" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="H711" s="2" t="s">
         <v>25</v>
@@ -46393,7 +46396,7 @@
         <v>622</v>
       </c>
       <c r="G712" s="2" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="H712" s="2" t="s">
         <v>24</v>
@@ -46452,7 +46455,7 @@
         <v>622</v>
       </c>
       <c r="G713" s="2" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="H713" s="2" t="s">
         <v>23</v>
@@ -46511,7 +46514,7 @@
         <v>622</v>
       </c>
       <c r="G714" s="2" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="H714" s="2" t="s">
         <v>21</v>
@@ -46570,7 +46573,7 @@
         <v>622</v>
       </c>
       <c r="G715" s="2" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="H715" s="2" t="s">
         <v>561</v>
@@ -46629,7 +46632,7 @@
         <v>622</v>
       </c>
       <c r="G716" s="2" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="H716" s="2" t="s">
         <v>25</v>
@@ -46688,7 +46691,7 @@
         <v>622</v>
       </c>
       <c r="G717" s="2" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="H717" s="2" t="s">
         <v>24</v>
@@ -46747,7 +46750,7 @@
         <v>622</v>
       </c>
       <c r="G718" s="2" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="H718" s="2" t="s">
         <v>23</v>
@@ -46806,7 +46809,7 @@
         <v>622</v>
       </c>
       <c r="G719" s="2" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="H719" s="2" t="s">
         <v>21</v>
@@ -46861,7 +46864,7 @@
       <c r="E720" s="2"/>
       <c r="F720" s="2"/>
       <c r="G720" s="2" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="H720" s="2" t="s">
         <v>124</v>
@@ -46916,7 +46919,7 @@
       <c r="E721" s="2"/>
       <c r="F721" s="2"/>
       <c r="G721" s="2" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="H721" s="2" t="s">
         <v>122</v>
@@ -46962,7 +46965,7 @@
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:T642">
     <sortCondition ref="A2:A642"/>
   </sortState>
-  <conditionalFormatting sqref="A1:T1 T1:U721 A2:F305 K2:K721 C306:C721 A493:B721 L651:L684 I653:J653 O653:T684 M654:N684 G660:J721 D661:F721 L685:T721">
+  <conditionalFormatting sqref="A1:T1 A2:F305 K2:K721 C306:C721 A493:B721 L651:L684 I653:J653 M654:N684 G660:J721 D661:F721 L685:T721 T1:U721 O653:T684">
     <cfRule type="expression" dxfId="12" priority="4">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
@@ -47012,12 +47015,12 @@
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L3:P303 S256:T301 Q294:R303 S302:S303 T302:T305 L304:S305 A306:B489 Q306:R565 L306:P626 S306:T642 D653:H660 G659:I659">
+  <conditionalFormatting sqref="L3:P303 S256:T301 Q294:R303 S302:S303 T302:T305 L304:S305 A306:B489 L306:P626 S306:T642 D653:H660 G659:I659 Q306:R565">
     <cfRule type="expression" dxfId="2" priority="27">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L2:T2 Q3:T255 Q256:R287 Q566:Q628 R566:R642 M629:Q630 L631:Q642 L643:T650 M651:T652">
+  <conditionalFormatting sqref="L2:T2 Q256:R287 Q566:Q628 R566:R642 M629:Q630 L631:Q642 L643:T650 M651:T652 Q3:T255">
     <cfRule type="expression" dxfId="1" priority="44">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>

</xml_diff>